<commit_message>
Added some new labels and linked datasets to datagroups.
</commit_message>
<xml_diff>
--- a/IEDC_content_fill/IEDC_Prototype_Datasets_Batch1_Upload_MASTER.xlsx
+++ b/IEDC_content_fill/IEDC_Prototype_Datasets_Batch1_Upload_MASTER.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Stefan Pauliuk\FILES\ARBEIT\PROJECTS\Database\IE_DataCommons\IEDC_software\IEDC_content_fill\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8580A113-F1BB-4BED-85CC-6465981B7080}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BC1FDE8-0C64-4F6C-89E9-91FF19A88D34}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="20448" windowHeight="9684" tabRatio="603" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17611" uniqueCount="3863">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18081" uniqueCount="4009">
   <si>
     <t>Description</t>
   </si>
@@ -11620,7 +11620,445 @@
     <t>table in supplement 1-s2.0-S2352550924000885-mmc2.xlsx, sheet "Material intensity of EV"</t>
   </si>
   <si>
-    <t>4 Sankey flow datasets</t>
+    <t>1_F_Economy_wide_MFA_Global_EU27_2005_HAAS</t>
+  </si>
+  <si>
+    <t>six aggregate economic processes: extraction, energy use, material use, final use (use phase), waste management, and recycling</t>
+  </si>
+  <si>
+    <t>all materials and commodities</t>
+  </si>
+  <si>
+    <t>4 MFA resource groups: biomass, fossil fuels, metals and metal ores, non-metallic minerals</t>
+  </si>
+  <si>
+    <t>Global and EU27</t>
+  </si>
+  <si>
+    <t>one global aggregate value and one aggregate value for the EU27 in 2005.</t>
+  </si>
+  <si>
+    <t>Sankey flow data for the economy-wide material flows by broad material category world-wide and in the EU in 2005, by HAAS et al. (2015).</t>
+  </si>
+  <si>
+    <t>economy-wide MFA; material flow accounting; circular economy; material cycle; Sankey; EU; EU27</t>
+  </si>
+  <si>
+    <t>Data are reported twice. Once on each material-type layer separately and once on the 'dry mass' layer to allow for drawing a Sankey that shows all layers at once. The waste rock flow (0.12 Gt/yr in the EU) is a separate flow and not included in the 'use as material' flow. This is a correction compared to the original Sankey diagram, which is why the material use and addition to stocks flows are 0.12 Gt/yr (EU27) smaller than originally reported.</t>
+  </si>
+  <si>
+    <t>Flow of all commodities from use as material to use phase in EU27 in 2005 measured as dry mass, all materials of all materials is 3.33 Gt/yr.</t>
+  </si>
+  <si>
+    <t>Willi HAAS</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1111/jiec.12244</t>
+  </si>
+  <si>
+    <t>spreadsheet, supplied by author</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Numbers supplied by main author and converted to IEDC templates. </t>
+  </si>
+  <si>
+    <t>SANKEY_LINK</t>
+  </si>
+  <si>
+    <t>1_F_Economy_wide_MFA_EU28_2014_MAYER</t>
+  </si>
+  <si>
+    <t>EU28</t>
+  </si>
+  <si>
+    <t>Aggregate value</t>
+  </si>
+  <si>
+    <t>Sankey flow data for the economy-wide material flows by broad material category in the EU in 2014, by MAYER et al. (2019).</t>
+  </si>
+  <si>
+    <t>economy-wide MFA; material flow accounting; circular economy; material cycle; Sankey; EU; EU28</t>
+  </si>
+  <si>
+    <t>Converted to IEDC template by reformatting data from sheet "All results" in jiec12809-sup-0002-suppmat.xlsx. Flow names were divided into material/commodity, origin process, and destination process. Data are reported twice. Once on each material-type layer separately and once on the 'dry mass' layer to allow for drawing a Sankey that shows all layers at once.</t>
+  </si>
+  <si>
+    <t>Flow of all commodities from use as material to use phase in EU28 in 2014 measured as mass, metal ores and metals of metal ores and metals is 178.39 Mt/yr.</t>
+  </si>
+  <si>
+    <t>Andreas MAYER</t>
+  </si>
+  <si>
+    <t>https://onlinelibrary.wiley.com/action/downloadSupplement?doi=10.1111%2Fjiec.12809&amp;file=jiec12809-sup-0002-SuppMat.xlsx</t>
+  </si>
+  <si>
+    <t>supplementary spreadsheet jiec12809-sup-0002-suppmat.xlsx</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1111/jiec.12809</t>
+  </si>
+  <si>
+    <t>Converted to IEDC template by reformatting data from sheet "All results" in jiec12809-sup-0002-suppmat.xlsx. Flow names were divided into material/commodity, origin process, and destination process.</t>
+  </si>
+  <si>
+    <t>1_F_Sand_Gravel_MFA_Global_184Countries_ZHUANG_2025</t>
+  </si>
+  <si>
+    <t>1_F_Watari_2025_SteelSankeys_30Regions</t>
+  </si>
+  <si>
+    <t>all stages of the steel cycle</t>
+  </si>
+  <si>
+    <t>aggregate industrial and consumer stages of the steel cycle</t>
+  </si>
+  <si>
+    <t>all broad iron-containing commodity groups in the steel cycle</t>
+  </si>
+  <si>
+    <t>from iron ore via steel, manufactured goods, end-of-life goods, to scrap</t>
+  </si>
+  <si>
+    <t>iron/steel</t>
+  </si>
+  <si>
+    <t>Individual values for 30 main producing countries</t>
+  </si>
+  <si>
+    <t>2000-2019</t>
+  </si>
+  <si>
+    <t>Sankey flow data for the steel cycle Sankeys by Takuma Watari et al. (2025)</t>
+  </si>
+  <si>
+    <t>steel; material cycle; Sankey; global</t>
+  </si>
+  <si>
+    <t>Numbers supplied by main author and converted to IEDC templates. For some processes, the balancing difference is indicated as 'mass balance gap'. The IEDC team did not check the mass balance of the reported data.</t>
+  </si>
+  <si>
+    <t>Flow of iron ore from mining to market for iron ore in China in 2000 measured as mass of iron is 63.42 Mt/yr.</t>
+  </si>
+  <si>
+    <t>https://github.com/takumawatari/steel-flows-sankey/tree/main/data</t>
+  </si>
+  <si>
+    <t>spreadsheet</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1016/j.resconrec.2025.108363</t>
+  </si>
+  <si>
+    <t>entry needs to be created first!</t>
+  </si>
+  <si>
+    <t>FutuRaM</t>
+  </si>
+  <si>
+    <t>https://futuram.eu/</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.6094/UNIFR/269286</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FutuRaM developed the Secondary Raw Materials knowledge base on the availability and recoverability of secondary raw materials (2RMs) within the European Union, with a special focus on critical raw materials (CRMs). </t>
+  </si>
+  <si>
+    <t>raw materials; secondary raw materials; urban mining; critical raw materials; circular economy;</t>
+  </si>
+  <si>
+    <t>FutuRaM_Database</t>
+  </si>
+  <si>
+    <t>Socio_metabolic_inequality_SMI</t>
+  </si>
+  <si>
+    <t>SMI_Lorenz_Curves</t>
+  </si>
+  <si>
+    <t>SMI_Indicators</t>
+  </si>
+  <si>
+    <t>Database of Lorenz curves, Gini cofficients, and other indicators for socio-metabolic inequality (inequality in service, stocks, and flows across society)</t>
+  </si>
+  <si>
+    <t>Inequality; socio-metabolic inequality; socio-economic metabolism; Lorenz curve; Gini index; Gini coefficient;</t>
+  </si>
+  <si>
+    <t>stocks, flows, and intensive product data (3_xxx)</t>
+  </si>
+  <si>
+    <t>in-use stocks, flows, and product material composition</t>
+  </si>
+  <si>
+    <t>many different authors and data suppliers, see the individual datasets</t>
+  </si>
+  <si>
+    <t>FutuRaM project consortium, see the individual datasets</t>
+  </si>
+  <si>
+    <t>Compilation of datasets from different sources</t>
+  </si>
+  <si>
+    <t>mass, units of products</t>
+  </si>
+  <si>
+    <t>main material cycle stages</t>
+  </si>
+  <si>
+    <t>manufacturing, use phase, waste management and recycling</t>
+  </si>
+  <si>
+    <t>major material uses</t>
+  </si>
+  <si>
+    <t>batteries, buildings, mining waste, slag and ashes, vehicles, WEEE, wind turbines</t>
+  </si>
+  <si>
+    <t>major material groups</t>
+  </si>
+  <si>
+    <t>Single country values</t>
+  </si>
+  <si>
+    <t>aluminium, iron, magnesium, steel, copper, concrete, plastics, zinc, critical raw materials</t>
+  </si>
+  <si>
+    <t>single year values, historic data til 2024 and future scenarios til 2050</t>
+  </si>
+  <si>
+    <t>stocks, flows, and intensive product properties</t>
+  </si>
+  <si>
+    <t>Lorenz curves for in-use stocks and flows (at scale) and normalized Lorenz curves (3_LC)</t>
+  </si>
+  <si>
+    <t>aggregrage processes</t>
+  </si>
+  <si>
+    <t>use phase (stock-flow-service nexus), entire economy</t>
+  </si>
+  <si>
+    <t>depends on dataset</t>
+  </si>
+  <si>
+    <t>all countries and regions, global</t>
+  </si>
+  <si>
+    <t>Different intensive and extensive indicators</t>
+  </si>
+  <si>
+    <t>Different intensive and extensive variables</t>
+  </si>
+  <si>
+    <t>Database of Lorenz curves for socio-metabolic inequality (inequality in service, stocks, and flows across society)</t>
+  </si>
+  <si>
+    <t>Database of Gini cofficients and other indicators for socio-metabolic inequality (inequality in service, stocks, and flows across society)</t>
+  </si>
+  <si>
+    <t>Inequality; socio-metabolic inequality; socio-economic metabolism; Lorenz curve;</t>
+  </si>
+  <si>
+    <t>Inequality; socio-metabolic inequality; socio-economic metabolism; Gini index; Gini coefficient;</t>
+  </si>
+  <si>
+    <t>see the individual datasets</t>
+  </si>
+  <si>
+    <t>POSTED</t>
+  </si>
+  <si>
+    <t>FutuRaM_Logos.png</t>
+  </si>
+  <si>
+    <t>Gini_DLS_1.png</t>
+  </si>
+  <si>
+    <t>https://github.com/PhilippVerpoort/posted</t>
+  </si>
+  <si>
+    <t>POSTED is a public database of techno-economic data on energy and climate-mitigation technologies and a framework for consistent handling of this database.</t>
+  </si>
+  <si>
+    <t>process data; industrial processes; industry technology; climate change mitigation; techno-economic data; unit process inventories; CAPEX; OPEX;</t>
+  </si>
+  <si>
+    <t>POSTED_industry_data</t>
+  </si>
+  <si>
+    <t>Philipp VERPOORT</t>
+  </si>
+  <si>
+    <t>POSTED_PIK_logo-light.png</t>
+  </si>
+  <si>
+    <t>Different intensive variables</t>
+  </si>
+  <si>
+    <t>unit process inventories, economic indicators (CAPEX, OPEX), lifetime</t>
+  </si>
+  <si>
+    <t>major industrial technologies</t>
+  </si>
+  <si>
+    <t>ca. 30 individual technologies and technology groups from the energy-intensive industry, such as cement production, steel production, or steam cracking</t>
+  </si>
+  <si>
+    <t>energy carriers</t>
+  </si>
+  <si>
+    <t>Aggregate values without explicit regional scope</t>
+  </si>
+  <si>
+    <t>single year values, depending on individual datasets</t>
+  </si>
+  <si>
+    <t>iTEM_Open_Transport_Data</t>
+  </si>
+  <si>
+    <t>https://transportenergy.org/open-data/</t>
+  </si>
+  <si>
+    <t>iTEM (International Transport Energy Modelling), a global group of researchers, is working to create a common, public, “best available” database of historical transport statistics for baseline calibration of models, through a transparent, scientific process.</t>
+  </si>
+  <si>
+    <t>transport; energy; vehicles; service; emissions;</t>
+  </si>
+  <si>
+    <t>iTEM team</t>
+  </si>
+  <si>
+    <t>iTEM_Logo.png</t>
+  </si>
+  <si>
+    <t>ca. 1970-2025-2100</t>
+  </si>
+  <si>
+    <t>single year values, historic data til 2024 and future scenarios til 2100</t>
+  </si>
+  <si>
+    <t>all major passenger and freight vehicle groups</t>
+  </si>
+  <si>
+    <t>use phase, manufacturing</t>
+  </si>
+  <si>
+    <t>in-use stocks, flows, service flows, emissions</t>
+  </si>
+  <si>
+    <t>6_MIP_Gini_Socio_Metabolic_Inequality_Collection</t>
+  </si>
+  <si>
+    <t>v1.0_April_2026</t>
+  </si>
+  <si>
+    <t>different focus processes, depends on the different data sources</t>
+  </si>
+  <si>
+    <t>depends on the different data sources</t>
+  </si>
+  <si>
+    <t>ca. 1970-2026</t>
+  </si>
+  <si>
+    <t>Compilation of Gini coeficients / Gini indices for socio-metabolic services, stocks, and flows, from different publications, see the comments for the individual entries in the dataset</t>
+  </si>
+  <si>
+    <t>Gini coefficient; Gini index; inequality; in-use stock; social metabolism; socio-metabolic inequality; provisioning systems; energy; materials; service;</t>
+  </si>
+  <si>
+    <t>Compilation of data from different publications, see the comments for the individual entries in the dataset</t>
+  </si>
+  <si>
+    <t>Value(E,I,g,p,r,t)</t>
+  </si>
+  <si>
+    <t>Gini index of final energy in/into/of/for residential buildings in use phase in Global in 2016 is 0.5838.</t>
+  </si>
+  <si>
+    <t>see the comments for the individual entries in the dataset</t>
+  </si>
+  <si>
+    <t>1_LCF_Final_Energy_Buildings_Vehicles_Global_PAULIUK_2024</t>
+  </si>
+  <si>
+    <t>Lorenz curve, non-normalized, flow</t>
+  </si>
+  <si>
+    <t>final energy for buildings and vehicles</t>
+  </si>
+  <si>
+    <t>all energy carriers for residential buildings, non-residential buildings, and passenger vehicles</t>
+  </si>
+  <si>
+    <t>one aggregate Lorenz curve</t>
+  </si>
+  <si>
+    <t>Lorenz curve for final energy for residential buildings, non-residential buildings, and passenger vehicles, based on region- and country-level data for 21 world regions</t>
+  </si>
+  <si>
+    <t>Value(g,r,t,o,d,1)</t>
+  </si>
+  <si>
+    <t>Lorenz curve, non-normalized, flow for final energy, all energy carriers from markets for final energy, all energy carriers to use phase - residential buildings in Global in 2016 for cumulative population share 0.79 is 16833561.656 TJ/yr.</t>
+  </si>
+  <si>
+    <t>[Data type] for [Aspect 1] from [Aspect 4] to [Aspect 5] in [Aspect 2] in [Aspect 3] for cumulative population share [Aspect 6] is [Value].</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1016/j.ecolecon.2024.108161</t>
+  </si>
+  <si>
+    <t>Lorenz curve; inequality; use phase; social metabolism; socio-metabolic inequality; provisioning systems; final energy; buildings; passenger vehicles;</t>
+  </si>
+  <si>
+    <t>Data extracted with Python script from supplementary data file Pauliuk_DLS_LorenzCurve_2024_SI.xlsx, sheet "pav_reb_nrb_Global_Fig4", converted to 1_LCF, and converted to IEDC templates. Cumulative population value rounded to two digits "0.xx".</t>
+  </si>
+  <si>
+    <t>Data extracted with Python script from supplementary data file, converted to 1_LCF, and converted to IEDC templates.</t>
+  </si>
+  <si>
+    <t>2_LCS_In_use_stock_Buildings_Vehicles_Global_PAULIUK_2024</t>
+  </si>
+  <si>
+    <t>Lorenz curve, non-normalized, stock</t>
+  </si>
+  <si>
+    <t>buildings and vehicles</t>
+  </si>
+  <si>
+    <t>residential buildings, non-residential buildings, and passenger vehicles</t>
+  </si>
+  <si>
+    <t>Lorenz curve for in-use stock of residential buildings, non-residential buildings, and passenger vehicles, based on region- and country-level data for 21 world regions</t>
+  </si>
+  <si>
+    <t>Lorenz curve; inequality; in-use stock; social metabolism; socio-metabolic inequality; provisioning systems; buildings; passenger vehicles;</t>
+  </si>
+  <si>
+    <t>Data extracted with Python script from supplementary data file Pauliuk_DLS_LorenzCurve_2024_SI.xlsx, sheet "pav_reb_nrb_Global_Fig4", converted to 2_LCS, and converted to IEDC templates. Cumulative population value rounded to two digits "0.xx".</t>
+  </si>
+  <si>
+    <t>Value(g,r,t,p,1)</t>
+  </si>
+  <si>
+    <t>Lorenz curve, non-normalized, stock for passenger vehicles in use phase - passenger vehicles in Global in 2015 for cumulative population share 0.32 is 39.495 million.</t>
+  </si>
+  <si>
+    <t>[Data type] for [Aspect 1] in [Aspect 4] in [Aspect 2] in [Aspect 3] for cumulative population share [Aspect 5] is [Value].</t>
+  </si>
+  <si>
+    <t>Data extracted with Python script from supplementary data file, converted to 2_LCS, and converted to IEDC templates.</t>
+  </si>
+  <si>
+    <t>needs correction, check IEDC-floweaver-Sankey workflow first</t>
+  </si>
+  <si>
+    <t>may need correction, check IEDC-floweaver-Sankey workflow first</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -11768,7 +12206,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -11844,12 +12282,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -12036,7 +12468,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="264">
+  <cellXfs count="267">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
@@ -12532,7 +12964,14 @@
     <xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
@@ -12542,8 +12981,8 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFC9A4E4"/>
       <color rgb="FFD3B5E9"/>
-      <color rgb="FFC9A4E4"/>
     </mruColors>
   </colors>
   <extLst>
@@ -12820,7 +13259,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:M32"/>
+  <dimension ref="B1:V32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.3" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="3" max="3" width="33" bestFit="1" customWidth="1"/>
@@ -12828,16 +13267,24 @@
     <col min="5" max="5" width="28.38671875" customWidth="1"/>
     <col min="6" max="6" width="17.6640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="17.88671875" customWidth="1"/>
+    <col min="14" max="15" width="10.6640625" style="105"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:13" x14ac:dyDescent="0.4">
+    <row r="1" spans="2:22" x14ac:dyDescent="0.4">
+      <c r="R1" s="105"/>
+      <c r="S1" s="105"/>
+      <c r="T1" s="105"/>
+      <c r="U1" s="105"/>
+      <c r="V1" s="105"/>
+    </row>
+    <row r="2" spans="2:22" x14ac:dyDescent="0.4">
       <c r="B2" s="34" t="s">
         <v>186</v>
       </c>
       <c r="C2" s="35"/>
       <c r="D2" s="35"/>
     </row>
-    <row r="3" spans="2:13" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:22" x14ac:dyDescent="0.4">
       <c r="B3" s="32"/>
       <c r="C3" s="31" t="s">
         <v>181</v>
@@ -12872,8 +13319,20 @@
       <c r="M3" s="39" t="s">
         <v>3448</v>
       </c>
+      <c r="N3" s="39" t="s">
+        <v>3912</v>
+      </c>
+      <c r="O3" s="39" t="s">
+        <v>3960</v>
+      </c>
+      <c r="P3" s="39" t="s">
+        <v>3906</v>
+      </c>
+      <c r="Q3" s="39" t="s">
+        <v>3944</v>
+      </c>
     </row>
-    <row r="4" spans="2:13" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:22" x14ac:dyDescent="0.4">
       <c r="B4" s="244" t="s">
         <v>2</v>
       </c>
@@ -12910,8 +13369,21 @@
       <c r="M4" s="140">
         <v>9</v>
       </c>
+      <c r="N4" s="140">
+        <v>10</v>
+      </c>
+      <c r="O4" s="140">
+        <v>11</v>
+      </c>
+      <c r="P4" s="140">
+        <v>12</v>
+      </c>
+      <c r="Q4" s="140">
+        <v>13</v>
+      </c>
+      <c r="R4" s="105"/>
     </row>
-    <row r="5" spans="2:13" x14ac:dyDescent="0.4">
+    <row r="5" spans="2:22" x14ac:dyDescent="0.4">
       <c r="B5" s="244"/>
       <c r="C5" s="26" t="s">
         <v>422</v>
@@ -12946,8 +13418,20 @@
       <c r="M5" s="118" t="s">
         <v>3448</v>
       </c>
+      <c r="N5" s="118" t="s">
+        <v>3912</v>
+      </c>
+      <c r="O5" s="118" t="s">
+        <v>3960</v>
+      </c>
+      <c r="P5" s="118" t="s">
+        <v>3906</v>
+      </c>
+      <c r="Q5" s="118" t="s">
+        <v>3944</v>
+      </c>
     </row>
-    <row r="6" spans="2:13" ht="13.3" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:22" ht="13.3" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B6" s="245" t="s">
         <v>6</v>
       </c>
@@ -12964,8 +13448,12 @@
       <c r="K6" s="121"/>
       <c r="L6" s="121"/>
       <c r="M6" s="121"/>
+      <c r="N6" s="121"/>
+      <c r="O6" s="121"/>
+      <c r="P6" s="121"/>
+      <c r="Q6" s="121"/>
     </row>
-    <row r="7" spans="2:13" x14ac:dyDescent="0.4">
+    <row r="7" spans="2:22" x14ac:dyDescent="0.4">
       <c r="B7" s="245"/>
       <c r="C7" s="26" t="s">
         <v>424</v>
@@ -12980,8 +13468,12 @@
       <c r="K7" s="121"/>
       <c r="L7" s="121"/>
       <c r="M7" s="121"/>
+      <c r="N7" s="121"/>
+      <c r="O7" s="121"/>
+      <c r="P7" s="121"/>
+      <c r="Q7" s="121"/>
     </row>
-    <row r="8" spans="2:13" x14ac:dyDescent="0.4">
+    <row r="8" spans="2:22" x14ac:dyDescent="0.4">
       <c r="B8" s="245"/>
       <c r="C8" s="26" t="s">
         <v>425</v>
@@ -12996,8 +13488,12 @@
       <c r="K8" s="121"/>
       <c r="L8" s="121"/>
       <c r="M8" s="121"/>
+      <c r="N8" s="121"/>
+      <c r="O8" s="121"/>
+      <c r="P8" s="121"/>
+      <c r="Q8" s="121"/>
     </row>
-    <row r="9" spans="2:13" x14ac:dyDescent="0.4">
+    <row r="9" spans="2:22" x14ac:dyDescent="0.4">
       <c r="B9" s="245"/>
       <c r="C9" s="28" t="s">
         <v>426</v>
@@ -13012,8 +13508,12 @@
       <c r="K9" s="121"/>
       <c r="L9" s="121"/>
       <c r="M9" s="121"/>
+      <c r="N9" s="121"/>
+      <c r="O9" s="121"/>
+      <c r="P9" s="121"/>
+      <c r="Q9" s="121"/>
     </row>
-    <row r="10" spans="2:13" x14ac:dyDescent="0.4">
+    <row r="10" spans="2:22" x14ac:dyDescent="0.4">
       <c r="B10" s="245"/>
       <c r="C10" s="27" t="s">
         <v>427</v>
@@ -13028,8 +13528,12 @@
       <c r="K10" s="121"/>
       <c r="L10" s="121"/>
       <c r="M10" s="121"/>
+      <c r="N10" s="121"/>
+      <c r="O10" s="121"/>
+      <c r="P10" s="121"/>
+      <c r="Q10" s="121"/>
     </row>
-    <row r="11" spans="2:13" x14ac:dyDescent="0.4">
+    <row r="11" spans="2:22" x14ac:dyDescent="0.4">
       <c r="B11" s="245"/>
       <c r="C11" s="27" t="s">
         <v>428</v>
@@ -13044,8 +13548,12 @@
       <c r="K11" s="121"/>
       <c r="L11" s="121"/>
       <c r="M11" s="121"/>
+      <c r="N11" s="121"/>
+      <c r="O11" s="121"/>
+      <c r="P11" s="121"/>
+      <c r="Q11" s="121"/>
     </row>
-    <row r="12" spans="2:13" x14ac:dyDescent="0.4">
+    <row r="12" spans="2:22" x14ac:dyDescent="0.4">
       <c r="B12" s="245"/>
       <c r="C12" s="27" t="s">
         <v>429</v>
@@ -13060,8 +13568,12 @@
       <c r="K12" s="121"/>
       <c r="L12" s="121"/>
       <c r="M12" s="121"/>
+      <c r="N12" s="121"/>
+      <c r="O12" s="121"/>
+      <c r="P12" s="121"/>
+      <c r="Q12" s="121"/>
     </row>
-    <row r="13" spans="2:13" x14ac:dyDescent="0.4">
+    <row r="13" spans="2:22" x14ac:dyDescent="0.4">
       <c r="B13" s="245"/>
       <c r="C13" s="27" t="s">
         <v>430</v>
@@ -13076,8 +13588,12 @@
       <c r="K13" s="121"/>
       <c r="L13" s="121"/>
       <c r="M13" s="121"/>
+      <c r="N13" s="121"/>
+      <c r="O13" s="121"/>
+      <c r="P13" s="121"/>
+      <c r="Q13" s="121"/>
     </row>
-    <row r="14" spans="2:13" x14ac:dyDescent="0.4">
+    <row r="14" spans="2:22" x14ac:dyDescent="0.4">
       <c r="B14" s="245"/>
       <c r="C14" s="27" t="s">
         <v>431</v>
@@ -13092,8 +13608,12 @@
       <c r="K14" s="121"/>
       <c r="L14" s="121"/>
       <c r="M14" s="121"/>
+      <c r="N14" s="121"/>
+      <c r="O14" s="121"/>
+      <c r="P14" s="121"/>
+      <c r="Q14" s="121"/>
     </row>
-    <row r="15" spans="2:13" x14ac:dyDescent="0.4">
+    <row r="15" spans="2:22" x14ac:dyDescent="0.4">
       <c r="B15" s="245"/>
       <c r="C15" s="27" t="s">
         <v>432</v>
@@ -13108,8 +13628,12 @@
       <c r="K15" s="121"/>
       <c r="L15" s="121"/>
       <c r="M15" s="121"/>
+      <c r="N15" s="121"/>
+      <c r="O15" s="121"/>
+      <c r="P15" s="121"/>
+      <c r="Q15" s="121"/>
     </row>
-    <row r="16" spans="2:13" x14ac:dyDescent="0.4">
+    <row r="16" spans="2:22" x14ac:dyDescent="0.4">
       <c r="B16" s="245"/>
       <c r="C16" s="27" t="s">
         <v>433</v>
@@ -13124,8 +13648,12 @@
       <c r="K16" s="121"/>
       <c r="L16" s="121"/>
       <c r="M16" s="121"/>
+      <c r="N16" s="121"/>
+      <c r="O16" s="121"/>
+      <c r="P16" s="121"/>
+      <c r="Q16" s="121"/>
     </row>
-    <row r="17" spans="2:13" x14ac:dyDescent="0.4">
+    <row r="17" spans="2:17" x14ac:dyDescent="0.4">
       <c r="B17" s="245"/>
       <c r="C17" s="27" t="s">
         <v>434</v>
@@ -13140,8 +13668,12 @@
       <c r="K17" s="121"/>
       <c r="L17" s="121"/>
       <c r="M17" s="121"/>
+      <c r="N17" s="121"/>
+      <c r="O17" s="121"/>
+      <c r="P17" s="121"/>
+      <c r="Q17" s="121"/>
     </row>
-    <row r="18" spans="2:13" x14ac:dyDescent="0.4">
+    <row r="18" spans="2:17" x14ac:dyDescent="0.4">
       <c r="B18" s="245"/>
       <c r="C18" s="27" t="s">
         <v>435</v>
@@ -13156,8 +13688,12 @@
       <c r="K18" s="121"/>
       <c r="L18" s="121"/>
       <c r="M18" s="121"/>
+      <c r="N18" s="121"/>
+      <c r="O18" s="121"/>
+      <c r="P18" s="121"/>
+      <c r="Q18" s="121"/>
     </row>
-    <row r="19" spans="2:13" x14ac:dyDescent="0.4">
+    <row r="19" spans="2:17" x14ac:dyDescent="0.4">
       <c r="B19" s="246" t="s">
         <v>0</v>
       </c>
@@ -13190,8 +13726,20 @@
       <c r="M19" s="118" t="s">
         <v>3450</v>
       </c>
+      <c r="N19" s="118" t="s">
+        <v>3915</v>
+      </c>
+      <c r="O19" s="118" t="s">
+        <v>3962</v>
+      </c>
+      <c r="P19" s="118" t="s">
+        <v>3909</v>
+      </c>
+      <c r="Q19" s="118" t="s">
+        <v>3948</v>
+      </c>
     </row>
-    <row r="20" spans="2:13" x14ac:dyDescent="0.4">
+    <row r="20" spans="2:17" x14ac:dyDescent="0.4">
       <c r="B20" s="246"/>
       <c r="C20" s="27" t="s">
         <v>437</v>
@@ -13226,8 +13774,20 @@
       <c r="M20" s="118" t="s">
         <v>3451</v>
       </c>
+      <c r="N20" s="118" t="s">
+        <v>3916</v>
+      </c>
+      <c r="O20" s="118" t="s">
+        <v>3963</v>
+      </c>
+      <c r="P20" s="118" t="s">
+        <v>3910</v>
+      </c>
+      <c r="Q20" s="118" t="s">
+        <v>3949</v>
+      </c>
     </row>
-    <row r="21" spans="2:13" x14ac:dyDescent="0.4">
+    <row r="21" spans="2:17" x14ac:dyDescent="0.4">
       <c r="B21" s="246"/>
       <c r="C21" s="27" t="s">
         <v>438</v>
@@ -13258,8 +13818,12 @@
       <c r="M21" s="118" t="s">
         <v>3452</v>
       </c>
+      <c r="N21" s="118"/>
+      <c r="O21" s="118"/>
+      <c r="P21" s="118"/>
+      <c r="Q21" s="118"/>
     </row>
-    <row r="22" spans="2:13" ht="13.3" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="22" spans="2:17" ht="13.3" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B22" s="247" t="s">
         <v>8</v>
       </c>
@@ -13294,8 +13858,20 @@
       <c r="M22" s="121" t="s">
         <v>860</v>
       </c>
+      <c r="N22" s="118" t="s">
+        <v>861</v>
+      </c>
+      <c r="O22" s="118" t="s">
+        <v>861</v>
+      </c>
+      <c r="P22" s="118" t="s">
+        <v>861</v>
+      </c>
+      <c r="Q22" s="118" t="s">
+        <v>861</v>
+      </c>
     </row>
-    <row r="23" spans="2:13" x14ac:dyDescent="0.4">
+    <row r="23" spans="2:17" x14ac:dyDescent="0.4">
       <c r="B23" s="247"/>
       <c r="C23" s="26" t="s">
         <v>440</v>
@@ -13310,8 +13886,12 @@
       <c r="K23" s="121"/>
       <c r="L23" s="121"/>
       <c r="M23" s="121"/>
+      <c r="N23" s="121"/>
+      <c r="O23" s="121"/>
+      <c r="P23" s="121"/>
+      <c r="Q23" s="121"/>
     </row>
-    <row r="24" spans="2:13" x14ac:dyDescent="0.4">
+    <row r="24" spans="2:17" x14ac:dyDescent="0.4">
       <c r="B24" s="247"/>
       <c r="C24" s="25" t="s">
         <v>441</v>
@@ -13326,8 +13906,12 @@
       <c r="K24" s="121"/>
       <c r="L24" s="121"/>
       <c r="M24" s="121"/>
+      <c r="N24" s="121"/>
+      <c r="O24" s="121"/>
+      <c r="P24" s="121"/>
+      <c r="Q24" s="121"/>
     </row>
-    <row r="25" spans="2:13" x14ac:dyDescent="0.4">
+    <row r="25" spans="2:17" x14ac:dyDescent="0.4">
       <c r="B25" s="247"/>
       <c r="C25" s="25" t="s">
         <v>443</v>
@@ -13358,8 +13942,20 @@
       <c r="M25" s="170" t="s">
         <v>3463</v>
       </c>
+      <c r="N25" s="170" t="s">
+        <v>3908</v>
+      </c>
+      <c r="O25" s="170" t="s">
+        <v>3961</v>
+      </c>
+      <c r="P25" s="170" t="s">
+        <v>3907</v>
+      </c>
+      <c r="Q25" s="170" t="s">
+        <v>3947</v>
+      </c>
     </row>
-    <row r="26" spans="2:13" x14ac:dyDescent="0.4">
+    <row r="26" spans="2:17" x14ac:dyDescent="0.4">
       <c r="B26" s="247"/>
       <c r="C26" s="25" t="s">
         <v>444</v>
@@ -13376,8 +13972,12 @@
       <c r="K26" s="121"/>
       <c r="L26" s="121"/>
       <c r="M26" s="121"/>
+      <c r="N26" s="121"/>
+      <c r="O26" s="121"/>
+      <c r="P26" s="121"/>
+      <c r="Q26" s="121"/>
     </row>
-    <row r="27" spans="2:13" x14ac:dyDescent="0.4">
+    <row r="27" spans="2:17" x14ac:dyDescent="0.4">
       <c r="B27" s="247"/>
       <c r="C27" s="25" t="s">
         <v>445</v>
@@ -13392,8 +13992,12 @@
       <c r="K27" s="121"/>
       <c r="L27" s="121"/>
       <c r="M27" s="121"/>
+      <c r="N27" s="121"/>
+      <c r="O27" s="121"/>
+      <c r="P27" s="121"/>
+      <c r="Q27" s="121"/>
     </row>
-    <row r="28" spans="2:13" ht="13.3" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="28" spans="2:17" ht="13.3" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B28" s="248" t="s">
         <v>9</v>
       </c>
@@ -13430,8 +14034,20 @@
       <c r="M28" s="180">
         <v>46020</v>
       </c>
+      <c r="N28" s="180">
+        <v>46031</v>
+      </c>
+      <c r="O28" s="180">
+        <v>46031</v>
+      </c>
+      <c r="P28" s="180">
+        <v>46031</v>
+      </c>
+      <c r="Q28" s="180">
+        <v>46031</v>
+      </c>
     </row>
-    <row r="29" spans="2:13" x14ac:dyDescent="0.4">
+    <row r="29" spans="2:17" x14ac:dyDescent="0.4">
       <c r="B29" s="248"/>
       <c r="C29" s="25" t="s">
         <v>447</v>
@@ -13466,8 +14082,20 @@
       <c r="M29" s="124" t="s">
         <v>30</v>
       </c>
+      <c r="N29" s="124" t="s">
+        <v>30</v>
+      </c>
+      <c r="O29" s="124" t="s">
+        <v>30</v>
+      </c>
+      <c r="P29" s="264" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q29" s="124" t="s">
+        <v>30</v>
+      </c>
     </row>
-    <row r="30" spans="2:13" x14ac:dyDescent="0.4">
+    <row r="30" spans="2:17" x14ac:dyDescent="0.4">
       <c r="B30" s="241" t="s">
         <v>185</v>
       </c>
@@ -13484,8 +14112,12 @@
       <c r="K30" s="181"/>
       <c r="L30" s="181"/>
       <c r="M30" s="181"/>
+      <c r="N30" s="181"/>
+      <c r="O30" s="181"/>
+      <c r="P30" s="181"/>
+      <c r="Q30" s="181"/>
     </row>
-    <row r="31" spans="2:13" x14ac:dyDescent="0.4">
+    <row r="31" spans="2:17" x14ac:dyDescent="0.4">
       <c r="B31" s="242"/>
       <c r="C31" s="108" t="s">
         <v>449</v>
@@ -13500,8 +14132,12 @@
       <c r="K31" s="164"/>
       <c r="L31" s="164"/>
       <c r="M31" s="164"/>
+      <c r="N31" s="164"/>
+      <c r="O31" s="164"/>
+      <c r="P31" s="164"/>
+      <c r="Q31" s="164"/>
     </row>
-    <row r="32" spans="2:13" x14ac:dyDescent="0.4">
+    <row r="32" spans="2:17" x14ac:dyDescent="0.4">
       <c r="B32" s="243"/>
       <c r="C32" s="109" t="s">
         <v>450</v>
@@ -13516,6 +14152,10 @@
       <c r="K32" s="166"/>
       <c r="L32" s="166"/>
       <c r="M32" s="166"/>
+      <c r="N32" s="166"/>
+      <c r="O32" s="166"/>
+      <c r="P32" s="166"/>
+      <c r="Q32" s="166"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -13532,7 +14172,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="B2:AJ39"/>
+  <dimension ref="B2:AO39"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.3" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="3" max="3" width="22.109375" bestFit="1" customWidth="1"/>
@@ -13554,9 +14194,10 @@
     <col min="22" max="22" width="40.71875" customWidth="1"/>
     <col min="23" max="23" width="32.6640625" customWidth="1"/>
     <col min="27" max="27" width="24.44140625" customWidth="1"/>
+    <col min="38" max="38" width="11.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:36" x14ac:dyDescent="0.4">
+    <row r="2" spans="2:41" x14ac:dyDescent="0.4">
       <c r="B2" s="34" t="s">
         <v>184</v>
       </c>
@@ -13573,7 +14214,7 @@
       <c r="AE2" s="105"/>
       <c r="AF2" s="105"/>
     </row>
-    <row r="3" spans="2:36" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:41" x14ac:dyDescent="0.4">
       <c r="B3" s="32"/>
       <c r="C3" s="17" t="s">
         <v>181</v>
@@ -13677,8 +14318,23 @@
       <c r="AJ3" s="82" t="s">
         <v>3491</v>
       </c>
+      <c r="AK3" s="82" t="s">
+        <v>3911</v>
+      </c>
+      <c r="AL3" s="82" t="s">
+        <v>3913</v>
+      </c>
+      <c r="AM3" s="82" t="s">
+        <v>3914</v>
+      </c>
+      <c r="AN3" s="82" t="s">
+        <v>3950</v>
+      </c>
+      <c r="AO3" s="82" t="s">
+        <v>3960</v>
+      </c>
     </row>
-    <row r="4" spans="2:36" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:41" x14ac:dyDescent="0.4">
       <c r="B4" s="249" t="s">
         <v>2</v>
       </c>
@@ -13784,8 +14440,23 @@
       <c r="AJ4" s="140">
         <v>32</v>
       </c>
+      <c r="AK4" s="140">
+        <v>33</v>
+      </c>
+      <c r="AL4" s="140">
+        <v>34</v>
+      </c>
+      <c r="AM4" s="140">
+        <v>35</v>
+      </c>
+      <c r="AN4" s="140">
+        <v>36</v>
+      </c>
+      <c r="AO4" s="140">
+        <v>37</v>
+      </c>
     </row>
-    <row r="5" spans="2:36" x14ac:dyDescent="0.4">
+    <row r="5" spans="2:41" x14ac:dyDescent="0.4">
       <c r="B5" s="250"/>
       <c r="C5" s="54" t="s">
         <v>452</v>
@@ -13889,8 +14560,23 @@
       <c r="AJ5" s="164" t="s">
         <v>3491</v>
       </c>
+      <c r="AK5" s="164" t="s">
+        <v>3911</v>
+      </c>
+      <c r="AL5" s="164" t="s">
+        <v>3913</v>
+      </c>
+      <c r="AM5" s="164" t="s">
+        <v>3914</v>
+      </c>
+      <c r="AN5" s="164" t="s">
+        <v>3950</v>
+      </c>
+      <c r="AO5" s="164" t="s">
+        <v>3960</v>
+      </c>
     </row>
-    <row r="6" spans="2:36" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:41" x14ac:dyDescent="0.4">
       <c r="B6" s="33"/>
       <c r="C6" s="54" t="s">
         <v>453</v>
@@ -13992,8 +14678,23 @@
       <c r="AJ6" s="164" t="s">
         <v>11</v>
       </c>
+      <c r="AK6" s="164" t="s">
+        <v>11</v>
+      </c>
+      <c r="AL6" s="164" t="s">
+        <v>11</v>
+      </c>
+      <c r="AM6" s="164" t="s">
+        <v>11</v>
+      </c>
+      <c r="AN6" s="164" t="s">
+        <v>11</v>
+      </c>
+      <c r="AO6" s="164" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="7" spans="2:36" x14ac:dyDescent="0.4">
+    <row r="7" spans="2:41" x14ac:dyDescent="0.4">
       <c r="B7" s="50" t="s">
         <v>3</v>
       </c>
@@ -14097,8 +14798,23 @@
       <c r="AJ7" s="164" t="s">
         <v>11</v>
       </c>
+      <c r="AK7" t="s">
+        <v>3906</v>
+      </c>
+      <c r="AL7" t="s">
+        <v>3912</v>
+      </c>
+      <c r="AM7" s="105" t="s">
+        <v>3912</v>
+      </c>
+      <c r="AN7" t="s">
+        <v>3944</v>
+      </c>
+      <c r="AO7" t="s">
+        <v>3960</v>
+      </c>
     </row>
-    <row r="8" spans="2:36" ht="13.3" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="2:41" ht="13.3" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B8" s="245" t="s">
         <v>6</v>
       </c>
@@ -14202,8 +14918,23 @@
       <c r="AJ8" s="23" t="s">
         <v>2574</v>
       </c>
+      <c r="AK8" s="23" t="s">
+        <v>3917</v>
+      </c>
+      <c r="AL8" s="23" t="s">
+        <v>3931</v>
+      </c>
+      <c r="AM8" s="23" t="s">
+        <v>3938</v>
+      </c>
+      <c r="AN8" s="23" t="s">
+        <v>3953</v>
+      </c>
+      <c r="AO8" s="23" t="s">
+        <v>3917</v>
+      </c>
     </row>
-    <row r="9" spans="2:36" x14ac:dyDescent="0.4">
+    <row r="9" spans="2:41" x14ac:dyDescent="0.4">
       <c r="B9" s="245"/>
       <c r="C9" s="54" t="s">
         <v>424</v>
@@ -14305,8 +15036,23 @@
       <c r="AJ9" s="23" t="s">
         <v>3492</v>
       </c>
+      <c r="AK9" s="23" t="s">
+        <v>3918</v>
+      </c>
+      <c r="AL9" s="23" t="s">
+        <v>3932</v>
+      </c>
+      <c r="AM9" s="23" t="s">
+        <v>3937</v>
+      </c>
+      <c r="AN9" s="23" t="s">
+        <v>3954</v>
+      </c>
+      <c r="AO9" s="23" t="s">
+        <v>3970</v>
+      </c>
     </row>
-    <row r="10" spans="2:36" x14ac:dyDescent="0.4">
+    <row r="10" spans="2:41" x14ac:dyDescent="0.4">
       <c r="B10" s="245"/>
       <c r="C10" s="54" t="s">
         <v>425</v>
@@ -14408,8 +15154,23 @@
       <c r="AJ10" s="23" t="s">
         <v>199</v>
       </c>
+      <c r="AK10" s="23" t="s">
+        <v>3922</v>
+      </c>
+      <c r="AL10" s="23" t="s">
+        <v>1025</v>
+      </c>
+      <c r="AM10" s="23" t="s">
+        <v>1091</v>
+      </c>
+      <c r="AN10" s="23" t="s">
+        <v>1091</v>
+      </c>
+      <c r="AO10" s="23" t="s">
+        <v>1025</v>
+      </c>
     </row>
-    <row r="11" spans="2:36" ht="13.8" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:41" ht="13.8" x14ac:dyDescent="0.45">
       <c r="B11" s="245"/>
       <c r="C11" s="55" t="s">
         <v>426</v>
@@ -14511,8 +15272,23 @@
       <c r="AJ11" s="23" t="s">
         <v>3493</v>
       </c>
+      <c r="AK11" s="23" t="s">
+        <v>3923</v>
+      </c>
+      <c r="AL11" s="23" t="s">
+        <v>3934</v>
+      </c>
+      <c r="AM11" s="23" t="s">
+        <v>3934</v>
+      </c>
+      <c r="AN11" s="23" t="s">
+        <v>782</v>
+      </c>
+      <c r="AO11" s="23" t="s">
+        <v>3969</v>
+      </c>
     </row>
-    <row r="12" spans="2:36" ht="13.8" x14ac:dyDescent="0.45">
+    <row r="12" spans="2:41" ht="13.8" x14ac:dyDescent="0.45">
       <c r="B12" s="245"/>
       <c r="C12" s="56" t="s">
         <v>427</v>
@@ -14614,8 +15390,23 @@
       <c r="AJ12" s="23" t="s">
         <v>3494</v>
       </c>
+      <c r="AK12" s="23" t="s">
+        <v>3924</v>
+      </c>
+      <c r="AL12" s="23" t="s">
+        <v>3933</v>
+      </c>
+      <c r="AM12" s="23" t="s">
+        <v>3933</v>
+      </c>
+      <c r="AN12" s="23" t="s">
+        <v>2274</v>
+      </c>
+      <c r="AO12" s="23" t="s">
+        <v>1995</v>
+      </c>
     </row>
-    <row r="13" spans="2:36" ht="13.8" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:41" ht="13.8" x14ac:dyDescent="0.45">
       <c r="B13" s="245"/>
       <c r="C13" s="56" t="s">
         <v>428</v>
@@ -14717,8 +15508,23 @@
       <c r="AJ13" s="23" t="s">
         <v>3347</v>
       </c>
+      <c r="AK13" s="23" t="s">
+        <v>3925</v>
+      </c>
+      <c r="AL13" s="23" t="s">
+        <v>1561</v>
+      </c>
+      <c r="AM13" s="23" t="s">
+        <v>1561</v>
+      </c>
+      <c r="AN13" s="23" t="s">
+        <v>3955</v>
+      </c>
+      <c r="AO13" s="23" t="s">
+        <v>597</v>
+      </c>
     </row>
-    <row r="14" spans="2:36" ht="13.8" x14ac:dyDescent="0.45">
+    <row r="14" spans="2:41" ht="13.8" x14ac:dyDescent="0.45">
       <c r="B14" s="245"/>
       <c r="C14" s="56" t="s">
         <v>429</v>
@@ -14820,8 +15626,23 @@
       <c r="AJ14" s="23" t="s">
         <v>3495</v>
       </c>
+      <c r="AK14" s="23" t="s">
+        <v>3926</v>
+      </c>
+      <c r="AL14" s="23" t="s">
+        <v>3935</v>
+      </c>
+      <c r="AM14" s="23" t="s">
+        <v>3935</v>
+      </c>
+      <c r="AN14" s="23" t="s">
+        <v>3956</v>
+      </c>
+      <c r="AO14" s="23" t="s">
+        <v>3968</v>
+      </c>
     </row>
-    <row r="15" spans="2:36" ht="13.8" x14ac:dyDescent="0.45">
+    <row r="15" spans="2:41" ht="13.8" x14ac:dyDescent="0.45">
       <c r="B15" s="245"/>
       <c r="C15" s="56" t="s">
         <v>430</v>
@@ -14923,8 +15744,23 @@
       <c r="AJ15" s="23" t="s">
         <v>3504</v>
       </c>
+      <c r="AK15" s="23" t="s">
+        <v>3927</v>
+      </c>
+      <c r="AL15" s="23" t="s">
+        <v>1679</v>
+      </c>
+      <c r="AM15" s="23" t="s">
+        <v>1679</v>
+      </c>
+      <c r="AN15" s="23" t="s">
+        <v>3957</v>
+      </c>
+      <c r="AO15" s="23" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="16" spans="2:36" ht="13.8" x14ac:dyDescent="0.45">
+    <row r="16" spans="2:41" ht="13.8" x14ac:dyDescent="0.45">
       <c r="B16" s="245"/>
       <c r="C16" s="56" t="s">
         <v>431</v>
@@ -15026,8 +15862,23 @@
       <c r="AJ16" s="23" t="s">
         <v>3503</v>
       </c>
+      <c r="AK16" s="23" t="s">
+        <v>3929</v>
+      </c>
+      <c r="AL16" s="23" t="s">
+        <v>3935</v>
+      </c>
+      <c r="AM16" s="23" t="s">
+        <v>3935</v>
+      </c>
+      <c r="AN16" s="23" t="s">
+        <v>2526</v>
+      </c>
+      <c r="AO16" s="23" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="17" spans="2:36" ht="13.8" x14ac:dyDescent="0.45">
+    <row r="17" spans="2:41" ht="13.8" x14ac:dyDescent="0.45">
       <c r="B17" s="245"/>
       <c r="C17" s="56" t="s">
         <v>432</v>
@@ -15129,8 +15980,23 @@
       <c r="AJ17" s="164" t="s">
         <v>156</v>
       </c>
+      <c r="AK17" s="164" t="s">
+        <v>1422</v>
+      </c>
+      <c r="AL17" s="164" t="s">
+        <v>3936</v>
+      </c>
+      <c r="AM17" s="164" t="s">
+        <v>3936</v>
+      </c>
+      <c r="AN17" s="164" t="s">
+        <v>19</v>
+      </c>
+      <c r="AO17" s="164" t="s">
+        <v>19</v>
+      </c>
     </row>
-    <row r="18" spans="2:36" ht="13.8" x14ac:dyDescent="0.45">
+    <row r="18" spans="2:41" ht="13.8" x14ac:dyDescent="0.45">
       <c r="B18" s="245"/>
       <c r="C18" s="56" t="s">
         <v>433</v>
@@ -15232,8 +16098,23 @@
       <c r="AJ18" s="164" t="s">
         <v>3502</v>
       </c>
+      <c r="AK18" s="164" t="s">
+        <v>3928</v>
+      </c>
+      <c r="AL18" s="23" t="s">
+        <v>3935</v>
+      </c>
+      <c r="AM18" s="23" t="s">
+        <v>3935</v>
+      </c>
+      <c r="AN18" s="164" t="s">
+        <v>3958</v>
+      </c>
+      <c r="AO18" s="164" t="s">
+        <v>3928</v>
+      </c>
     </row>
-    <row r="19" spans="2:36" x14ac:dyDescent="0.4">
+    <row r="19" spans="2:41" x14ac:dyDescent="0.4">
       <c r="B19" s="245"/>
       <c r="C19" s="56" t="s">
         <v>434</v>
@@ -15335,8 +16216,23 @@
       <c r="AJ19" s="23" t="s">
         <v>3498</v>
       </c>
+      <c r="AK19" s="23" t="s">
+        <v>1891</v>
+      </c>
+      <c r="AL19" s="23" t="s">
+        <v>3046</v>
+      </c>
+      <c r="AM19" s="23" t="s">
+        <v>3046</v>
+      </c>
+      <c r="AN19" s="23" t="s">
+        <v>3511</v>
+      </c>
+      <c r="AO19" s="23" t="s">
+        <v>3966</v>
+      </c>
     </row>
-    <row r="20" spans="2:36" ht="13.8" x14ac:dyDescent="0.45">
+    <row r="20" spans="2:41" ht="13.8" x14ac:dyDescent="0.45">
       <c r="B20" s="245"/>
       <c r="C20" s="56" t="s">
         <v>435</v>
@@ -15438,8 +16334,23 @@
       <c r="AJ20" s="164" t="s">
         <v>3499</v>
       </c>
+      <c r="AK20" s="164" t="s">
+        <v>3930</v>
+      </c>
+      <c r="AL20" s="23" t="s">
+        <v>3935</v>
+      </c>
+      <c r="AM20" s="23" t="s">
+        <v>3935</v>
+      </c>
+      <c r="AN20" s="164" t="s">
+        <v>3959</v>
+      </c>
+      <c r="AO20" s="164" t="s">
+        <v>3967</v>
+      </c>
     </row>
-    <row r="21" spans="2:36" ht="13.8" x14ac:dyDescent="0.45">
+    <row r="21" spans="2:41" ht="13.8" x14ac:dyDescent="0.45">
       <c r="B21" s="246" t="s">
         <v>0</v>
       </c>
@@ -15543,8 +16454,23 @@
       <c r="AJ21" s="23" t="s">
         <v>3500</v>
       </c>
+      <c r="AK21" s="23" t="s">
+        <v>3909</v>
+      </c>
+      <c r="AL21" s="23" t="s">
+        <v>3939</v>
+      </c>
+      <c r="AM21" s="23" t="s">
+        <v>3940</v>
+      </c>
+      <c r="AN21" s="23" t="s">
+        <v>3948</v>
+      </c>
+      <c r="AO21" s="23" t="s">
+        <v>3962</v>
+      </c>
     </row>
-    <row r="22" spans="2:36" ht="13.8" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:41" ht="13.8" x14ac:dyDescent="0.45">
       <c r="B22" s="246"/>
       <c r="C22" s="56" t="s">
         <v>437</v>
@@ -15648,8 +16574,23 @@
       <c r="AJ22" s="164" t="s">
         <v>3501</v>
       </c>
+      <c r="AK22" s="164" t="s">
+        <v>3910</v>
+      </c>
+      <c r="AL22" s="164" t="s">
+        <v>3941</v>
+      </c>
+      <c r="AM22" s="164" t="s">
+        <v>3942</v>
+      </c>
+      <c r="AN22" s="164" t="s">
+        <v>3949</v>
+      </c>
+      <c r="AO22" s="164" t="s">
+        <v>3963</v>
+      </c>
     </row>
-    <row r="23" spans="2:36" x14ac:dyDescent="0.4">
+    <row r="23" spans="2:41" x14ac:dyDescent="0.4">
       <c r="B23" s="246"/>
       <c r="C23" s="56" t="s">
         <v>454</v>
@@ -15741,8 +16682,23 @@
       <c r="AH23" s="164"/>
       <c r="AI23" s="164"/>
       <c r="AJ23" s="164"/>
+      <c r="AK23" s="164" t="s">
+        <v>3945</v>
+      </c>
+      <c r="AL23" s="164" t="s">
+        <v>3946</v>
+      </c>
+      <c r="AM23" s="164" t="s">
+        <v>3946</v>
+      </c>
+      <c r="AN23" s="164" t="s">
+        <v>3952</v>
+      </c>
+      <c r="AO23" s="164" t="s">
+        <v>3965</v>
+      </c>
     </row>
-    <row r="24" spans="2:36" ht="13.8" x14ac:dyDescent="0.45">
+    <row r="24" spans="2:41" ht="13.8" x14ac:dyDescent="0.45">
       <c r="B24" s="246"/>
       <c r="C24" s="56" t="s">
         <v>438</v>
@@ -15830,8 +16786,17 @@
         <v>3487</v>
       </c>
       <c r="AJ24" s="164"/>
+      <c r="AK24" s="164"/>
+      <c r="AL24" s="164" t="s">
+        <v>3921</v>
+      </c>
+      <c r="AM24" s="164" t="s">
+        <v>3921</v>
+      </c>
+      <c r="AN24" s="164"/>
+      <c r="AO24" s="164"/>
     </row>
-    <row r="25" spans="2:36" ht="13.3" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:41" ht="13.3" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B25" s="247" t="s">
         <v>8</v>
       </c>
@@ -15935,8 +16900,23 @@
       <c r="AJ25" s="23" t="s">
         <v>206</v>
       </c>
+      <c r="AK25" s="23" t="s">
+        <v>861</v>
+      </c>
+      <c r="AL25" s="23" t="s">
+        <v>206</v>
+      </c>
+      <c r="AM25" s="23" t="s">
+        <v>206</v>
+      </c>
+      <c r="AN25" s="23" t="s">
+        <v>861</v>
+      </c>
+      <c r="AO25" s="23" t="s">
+        <v>861</v>
+      </c>
     </row>
-    <row r="26" spans="2:36" x14ac:dyDescent="0.4">
+    <row r="26" spans="2:41" x14ac:dyDescent="0.4">
       <c r="B26" s="247"/>
       <c r="C26" s="54" t="s">
         <v>440</v>
@@ -16038,8 +17018,23 @@
       <c r="AJ26" s="164" t="s">
         <v>3109</v>
       </c>
+      <c r="AK26" s="164" t="s">
+        <v>2651</v>
+      </c>
+      <c r="AL26" s="164" t="s">
+        <v>2651</v>
+      </c>
+      <c r="AM26" s="164" t="s">
+        <v>2651</v>
+      </c>
+      <c r="AN26" s="164" t="s">
+        <v>61</v>
+      </c>
+      <c r="AO26" s="164" t="s">
+        <v>2651</v>
+      </c>
     </row>
-    <row r="27" spans="2:36" x14ac:dyDescent="0.4">
+    <row r="27" spans="2:41" x14ac:dyDescent="0.4">
       <c r="B27" s="247"/>
       <c r="C27" s="13" t="s">
         <v>441</v>
@@ -16141,8 +17136,23 @@
       <c r="AJ27" s="164" t="s">
         <v>3497</v>
       </c>
+      <c r="AK27" s="164" t="s">
+        <v>3920</v>
+      </c>
+      <c r="AL27" s="164" t="s">
+        <v>3919</v>
+      </c>
+      <c r="AM27" s="164" t="s">
+        <v>3919</v>
+      </c>
+      <c r="AN27" s="164" t="s">
+        <v>3951</v>
+      </c>
+      <c r="AO27" s="164" t="s">
+        <v>3964</v>
+      </c>
     </row>
-    <row r="28" spans="2:36" x14ac:dyDescent="0.4">
+    <row r="28" spans="2:41" x14ac:dyDescent="0.4">
       <c r="B28" s="247"/>
       <c r="C28" s="13" t="s">
         <v>443</v>
@@ -16244,8 +17254,23 @@
       <c r="AJ28" s="179" t="s">
         <v>3496</v>
       </c>
+      <c r="AK28" s="170" t="s">
+        <v>3907</v>
+      </c>
+      <c r="AL28" s="170" t="s">
+        <v>3908</v>
+      </c>
+      <c r="AM28" s="170" t="s">
+        <v>3908</v>
+      </c>
+      <c r="AN28" s="170" t="s">
+        <v>3947</v>
+      </c>
+      <c r="AO28" s="170" t="s">
+        <v>3961</v>
+      </c>
     </row>
-    <row r="29" spans="2:36" ht="13.8" x14ac:dyDescent="0.45">
+    <row r="29" spans="2:41" ht="13.8" x14ac:dyDescent="0.45">
       <c r="B29" s="247"/>
       <c r="C29" s="13" t="s">
         <v>444</v>
@@ -16347,8 +17372,23 @@
       <c r="AJ29" s="179" t="s">
         <v>3496</v>
       </c>
+      <c r="AK29" s="170" t="s">
+        <v>3907</v>
+      </c>
+      <c r="AL29" s="179" t="s">
+        <v>2225</v>
+      </c>
+      <c r="AM29" s="179" t="s">
+        <v>2225</v>
+      </c>
+      <c r="AN29" s="170" t="s">
+        <v>3947</v>
+      </c>
+      <c r="AO29" s="170" t="s">
+        <v>3961</v>
+      </c>
     </row>
-    <row r="30" spans="2:36" ht="13.8" x14ac:dyDescent="0.45">
+    <row r="30" spans="2:41" ht="13.8" x14ac:dyDescent="0.45">
       <c r="B30" s="247"/>
       <c r="C30" s="13" t="s">
         <v>445</v>
@@ -16450,8 +17490,23 @@
       <c r="AJ30" s="179" t="s">
         <v>3496</v>
       </c>
+      <c r="AK30" s="170" t="s">
+        <v>3907</v>
+      </c>
+      <c r="AL30" s="179" t="s">
+        <v>3943</v>
+      </c>
+      <c r="AM30" s="179" t="s">
+        <v>3943</v>
+      </c>
+      <c r="AN30" s="170" t="s">
+        <v>3947</v>
+      </c>
+      <c r="AO30" s="170" t="s">
+        <v>3961</v>
+      </c>
     </row>
-    <row r="31" spans="2:36" ht="13.3" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="31" spans="2:41" ht="13.3" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B31" s="248" t="s">
         <v>9</v>
       </c>
@@ -16557,8 +17612,23 @@
       <c r="AJ31" s="161">
         <v>46024</v>
       </c>
+      <c r="AK31" s="161">
+        <v>46031</v>
+      </c>
+      <c r="AL31" s="161">
+        <v>46031</v>
+      </c>
+      <c r="AM31" s="161">
+        <v>46031</v>
+      </c>
+      <c r="AN31" s="161">
+        <v>46031</v>
+      </c>
+      <c r="AO31" s="161">
+        <v>46031</v>
+      </c>
     </row>
-    <row r="32" spans="2:36" x14ac:dyDescent="0.4">
+    <row r="32" spans="2:41" x14ac:dyDescent="0.4">
       <c r="B32" s="251"/>
       <c r="C32" s="86" t="s">
         <v>447</v>
@@ -16662,8 +17732,23 @@
       <c r="AJ32" s="164" t="s">
         <v>30</v>
       </c>
+      <c r="AK32" s="164" t="s">
+        <v>30</v>
+      </c>
+      <c r="AL32" s="164" t="s">
+        <v>30</v>
+      </c>
+      <c r="AM32" s="164" t="s">
+        <v>30</v>
+      </c>
+      <c r="AN32" s="164" t="s">
+        <v>30</v>
+      </c>
+      <c r="AO32" s="164" t="s">
+        <v>30</v>
+      </c>
     </row>
-    <row r="33" spans="2:36" x14ac:dyDescent="0.4">
+    <row r="33" spans="2:41" x14ac:dyDescent="0.4">
       <c r="B33" s="241" t="s">
         <v>185</v>
       </c>
@@ -16703,8 +17788,13 @@
       <c r="AH33" s="164"/>
       <c r="AI33" s="164"/>
       <c r="AJ33" s="164"/>
+      <c r="AK33" s="164"/>
+      <c r="AL33" s="164"/>
+      <c r="AM33" s="164"/>
+      <c r="AN33" s="164"/>
+      <c r="AO33" s="164"/>
     </row>
-    <row r="34" spans="2:36" x14ac:dyDescent="0.4">
+    <row r="34" spans="2:41" x14ac:dyDescent="0.4">
       <c r="B34" s="242"/>
       <c r="C34" s="15" t="s">
         <v>449</v>
@@ -16742,8 +17832,13 @@
       <c r="AH34" s="164"/>
       <c r="AI34" s="164"/>
       <c r="AJ34" s="164"/>
+      <c r="AK34" s="164"/>
+      <c r="AL34" s="164"/>
+      <c r="AM34" s="164"/>
+      <c r="AN34" s="164"/>
+      <c r="AO34" s="164"/>
     </row>
-    <row r="35" spans="2:36" x14ac:dyDescent="0.4">
+    <row r="35" spans="2:41" x14ac:dyDescent="0.4">
       <c r="B35" s="243"/>
       <c r="C35" s="16" t="s">
         <v>450</v>
@@ -16781,11 +17876,16 @@
       <c r="AH35" s="166"/>
       <c r="AI35" s="166"/>
       <c r="AJ35" s="166"/>
+      <c r="AK35" s="166"/>
+      <c r="AL35" s="166"/>
+      <c r="AM35" s="166"/>
+      <c r="AN35" s="166"/>
+      <c r="AO35" s="166"/>
     </row>
-    <row r="36" spans="2:36" x14ac:dyDescent="0.4">
+    <row r="36" spans="2:41" x14ac:dyDescent="0.4">
       <c r="W36" s="105"/>
     </row>
-    <row r="39" spans="2:36" x14ac:dyDescent="0.4">
+    <row r="39" spans="2:41" x14ac:dyDescent="0.4">
       <c r="I39" s="12"/>
     </row>
   </sheetData>
@@ -16870,7 +17970,7 @@
     <col min="239" max="16384" width="11.5546875" style="41"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:257" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:260" x14ac:dyDescent="0.4">
       <c r="C1" s="73" t="s">
         <v>269</v>
       </c>
@@ -17431,20 +18531,17 @@
       <c r="IQ1" s="174"/>
       <c r="IR1" s="174"/>
       <c r="IS1" s="174"/>
-      <c r="IT1" s="263" t="s">
-        <v>3862</v>
-      </c>
-      <c r="IU1" s="263" t="s">
-        <v>3862</v>
-      </c>
-      <c r="IV1" s="263" t="s">
-        <v>3862</v>
-      </c>
-      <c r="IW1" s="263" t="s">
-        <v>3862</v>
-      </c>
+      <c r="IT1" s="174"/>
+      <c r="IU1" s="174"/>
+      <c r="IV1" s="174"/>
+      <c r="IW1" s="233" t="s">
+        <v>3905</v>
+      </c>
+      <c r="IX1" s="174"/>
+      <c r="IY1" s="174"/>
+      <c r="IZ1" s="174"/>
     </row>
-    <row r="2" spans="1:257" ht="13.8" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:260" ht="13.8" x14ac:dyDescent="0.45">
       <c r="B2" s="34" t="s">
         <v>183</v>
       </c>
@@ -17938,6 +19035,9 @@
       <c r="HR2" s="154" t="s">
         <v>3846</v>
       </c>
+      <c r="HS2" s="233" t="s">
+        <v>3845</v>
+      </c>
       <c r="HT2" s="154" t="s">
         <v>3846</v>
       </c>
@@ -17953,6 +19053,9 @@
       <c r="HX2" s="154" t="s">
         <v>3846</v>
       </c>
+      <c r="HY2" s="233" t="s">
+        <v>3845</v>
+      </c>
       <c r="HZ2" s="154" t="s">
         <v>3846</v>
       </c>
@@ -18013,12 +19116,29 @@
       <c r="IS2" s="154" t="s">
         <v>3846</v>
       </c>
-      <c r="IT2" s="263"/>
-      <c r="IU2" s="263"/>
-      <c r="IV2" s="263"/>
-      <c r="IW2" s="263"/>
+      <c r="IT2" s="154" t="s">
+        <v>3846</v>
+      </c>
+      <c r="IU2" s="154" t="s">
+        <v>3846</v>
+      </c>
+      <c r="IV2" s="154" t="s">
+        <v>3846</v>
+      </c>
+      <c r="IW2" s="233" t="s">
+        <v>3845</v>
+      </c>
+      <c r="IX2" s="233" t="s">
+        <v>3845</v>
+      </c>
+      <c r="IY2" s="154" t="s">
+        <v>3846</v>
+      </c>
+      <c r="IZ2" s="154" t="s">
+        <v>3846</v>
+      </c>
     </row>
-    <row r="3" spans="1:257" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:260" x14ac:dyDescent="0.4">
       <c r="B3" s="58"/>
       <c r="C3" s="17" t="s">
         <v>181</v>
@@ -18272,15 +19392,24 @@
       <c r="DT3" s="105"/>
       <c r="HN3" s="105"/>
       <c r="HO3" s="105"/>
-      <c r="HS3" s="233" t="s">
-        <v>3845</v>
-      </c>
       <c r="HT3" s="105"/>
-      <c r="HY3" s="233" t="s">
-        <v>3845</v>
+      <c r="IK3" s="265" t="s">
+        <v>4006</v>
+      </c>
+      <c r="IT3" s="233" t="s">
+        <v>4007</v>
+      </c>
+      <c r="IU3" s="233" t="s">
+        <v>4007</v>
+      </c>
+      <c r="IV3" s="233" t="s">
+        <v>4007</v>
+      </c>
+      <c r="IW3" s="266" t="s">
+        <v>4008</v>
       </c>
     </row>
-    <row r="4" spans="1:257" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:260" x14ac:dyDescent="0.4">
       <c r="A4" s="41">
         <v>1</v>
       </c>
@@ -18538,7 +19667,7 @@
       <c r="DS4" s="105"/>
       <c r="DT4" s="105"/>
     </row>
-    <row r="5" spans="1:257" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:260" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="41">
         <v>2</v>
       </c>
@@ -19296,8 +20425,29 @@
       <c r="IS5" s="115" t="s">
         <v>3847</v>
       </c>
+      <c r="IT5" s="115" t="s">
+        <v>3862</v>
+      </c>
+      <c r="IU5" s="115" t="s">
+        <v>3877</v>
+      </c>
+      <c r="IV5" s="115" t="s">
+        <v>3890</v>
+      </c>
+      <c r="IW5" s="105" t="s">
+        <v>3889</v>
+      </c>
+      <c r="IX5" s="115" t="s">
+        <v>3971</v>
+      </c>
+      <c r="IY5" s="115" t="s">
+        <v>3982</v>
+      </c>
+      <c r="IZ5" s="115" t="s">
+        <v>3995</v>
+      </c>
     </row>
-    <row r="6" spans="1:257" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:260" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="92">
         <v>3</v>
       </c>
@@ -20053,8 +21203,26 @@
       <c r="IS6" s="115" t="s">
         <v>11</v>
       </c>
+      <c r="IT6" s="115" t="s">
+        <v>11</v>
+      </c>
+      <c r="IU6" s="115" t="s">
+        <v>11</v>
+      </c>
+      <c r="IV6" s="115" t="s">
+        <v>11</v>
+      </c>
+      <c r="IX6" s="263" t="s">
+        <v>3972</v>
+      </c>
+      <c r="IY6" s="115" t="s">
+        <v>11</v>
+      </c>
+      <c r="IZ6" s="115" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="7" spans="1:257" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:260" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="92">
         <v>4</v>
       </c>
@@ -20812,8 +21980,26 @@
       <c r="IS7" s="115" t="s">
         <v>845</v>
       </c>
+      <c r="IT7" s="115" t="s">
+        <v>845</v>
+      </c>
+      <c r="IU7" s="115" t="s">
+        <v>845</v>
+      </c>
+      <c r="IV7" s="115" t="s">
+        <v>845</v>
+      </c>
+      <c r="IX7" s="115">
+        <v>35</v>
+      </c>
+      <c r="IY7" s="115">
+        <v>34</v>
+      </c>
+      <c r="IZ7" s="115">
+        <v>34</v>
+      </c>
     </row>
-    <row r="8" spans="1:257" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:260" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="92">
         <v>5</v>
       </c>
@@ -21571,8 +22757,26 @@
       <c r="IS8" s="115">
         <v>3</v>
       </c>
+      <c r="IT8" s="115">
+        <v>1</v>
+      </c>
+      <c r="IU8" s="115">
+        <v>1</v>
+      </c>
+      <c r="IV8" s="115">
+        <v>1</v>
+      </c>
+      <c r="IX8" s="115">
+        <v>6</v>
+      </c>
+      <c r="IY8" s="115">
+        <v>1</v>
+      </c>
+      <c r="IZ8" s="115">
+        <v>2</v>
+      </c>
     </row>
-    <row r="9" spans="1:257" ht="28.2" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:260" ht="28.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="92">
         <v>6</v>
       </c>
@@ -22330,8 +23534,26 @@
       <c r="IS9" s="115" t="s">
         <v>846</v>
       </c>
+      <c r="IT9" s="115" t="s">
+        <v>1</v>
+      </c>
+      <c r="IU9" s="115" t="s">
+        <v>1</v>
+      </c>
+      <c r="IV9" s="115" t="s">
+        <v>1</v>
+      </c>
+      <c r="IX9" s="115" t="s">
+        <v>1676</v>
+      </c>
+      <c r="IY9" s="115" t="s">
+        <v>3983</v>
+      </c>
+      <c r="IZ9" s="115" t="s">
+        <v>3996</v>
+      </c>
     </row>
-    <row r="10" spans="1:257" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:260" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="92">
         <v>7</v>
       </c>
@@ -23089,8 +24311,26 @@
       <c r="IS10" s="115" t="s">
         <v>824</v>
       </c>
+      <c r="IT10" s="115" t="s">
+        <v>2007</v>
+      </c>
+      <c r="IU10" s="115" t="s">
+        <v>2007</v>
+      </c>
+      <c r="IV10" s="115" t="s">
+        <v>12</v>
+      </c>
+      <c r="IX10" s="115" t="s">
+        <v>3613</v>
+      </c>
+      <c r="IY10" s="115" t="s">
+        <v>3018</v>
+      </c>
+      <c r="IZ10" s="115" t="s">
+        <v>1025</v>
+      </c>
     </row>
-    <row r="11" spans="1:257" ht="14.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:260" ht="14.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="92">
         <v>8</v>
       </c>
@@ -23848,8 +25088,26 @@
       <c r="IS11" s="115" t="s">
         <v>782</v>
       </c>
+      <c r="IT11" s="115" t="s">
+        <v>1677</v>
+      </c>
+      <c r="IU11" s="115" t="s">
+        <v>1677</v>
+      </c>
+      <c r="IV11" s="115" t="s">
+        <v>3891</v>
+      </c>
+      <c r="IX11" s="115" t="s">
+        <v>1460</v>
+      </c>
+      <c r="IY11" s="115" t="s">
+        <v>782</v>
+      </c>
+      <c r="IZ11" s="115" t="s">
+        <v>782</v>
+      </c>
     </row>
-    <row r="12" spans="1:257" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:260" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="92">
         <v>9</v>
       </c>
@@ -24605,8 +25863,26 @@
       <c r="IS12" s="115" t="s">
         <v>2274</v>
       </c>
+      <c r="IT12" s="115" t="s">
+        <v>3863</v>
+      </c>
+      <c r="IU12" s="115" t="s">
+        <v>3863</v>
+      </c>
+      <c r="IV12" s="115" t="s">
+        <v>3892</v>
+      </c>
+      <c r="IX12" s="115" t="s">
+        <v>3973</v>
+      </c>
+      <c r="IY12" s="115" t="s">
+        <v>2274</v>
+      </c>
+      <c r="IZ12" s="115" t="s">
+        <v>2274</v>
+      </c>
     </row>
-    <row r="13" spans="1:257" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:260" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="92">
         <v>10</v>
       </c>
@@ -25362,8 +26638,26 @@
       <c r="IS13" s="115" t="s">
         <v>816</v>
       </c>
+      <c r="IT13" s="115" t="s">
+        <v>3864</v>
+      </c>
+      <c r="IU13" s="115" t="s">
+        <v>3864</v>
+      </c>
+      <c r="IV13" s="115" t="s">
+        <v>3893</v>
+      </c>
+      <c r="IX13" s="115" t="s">
+        <v>3568</v>
+      </c>
+      <c r="IY13" s="115" t="s">
+        <v>3984</v>
+      </c>
+      <c r="IZ13" s="115" t="s">
+        <v>3997</v>
+      </c>
     </row>
-    <row r="14" spans="1:257" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:260" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="92">
         <v>11</v>
       </c>
@@ -26119,8 +27413,26 @@
       <c r="IS14" s="115" t="s">
         <v>3848</v>
       </c>
+      <c r="IT14" s="115" t="s">
+        <v>3865</v>
+      </c>
+      <c r="IU14" s="115" t="s">
+        <v>3865</v>
+      </c>
+      <c r="IV14" s="115" t="s">
+        <v>3894</v>
+      </c>
+      <c r="IX14" s="115" t="s">
+        <v>3974</v>
+      </c>
+      <c r="IY14" s="115" t="s">
+        <v>3985</v>
+      </c>
+      <c r="IZ14" s="115" t="s">
+        <v>3998</v>
+      </c>
     </row>
-    <row r="15" spans="1:257" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="1:260" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="92">
         <v>12</v>
       </c>
@@ -26876,8 +28188,26 @@
       <c r="IS15" s="115" t="s">
         <v>3849</v>
       </c>
+      <c r="IT15" s="115" t="s">
+        <v>3864</v>
+      </c>
+      <c r="IU15" s="115" t="s">
+        <v>3864</v>
+      </c>
+      <c r="IV15" s="115" t="s">
+        <v>3895</v>
+      </c>
+      <c r="IX15" s="115" t="s">
+        <v>11</v>
+      </c>
+      <c r="IY15" s="115" t="s">
+        <v>11</v>
+      </c>
+      <c r="IZ15" s="115" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="16" spans="1:257" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:260" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="92">
         <v>13</v>
       </c>
@@ -27633,8 +28963,26 @@
       <c r="IS16" s="115" t="s">
         <v>3850</v>
       </c>
+      <c r="IT16" s="115" t="s">
+        <v>3865</v>
+      </c>
+      <c r="IU16" s="115" t="s">
+        <v>3865</v>
+      </c>
+      <c r="IV16" s="115" t="s">
+        <v>1680</v>
+      </c>
+      <c r="IX16" s="115" t="s">
+        <v>11</v>
+      </c>
+      <c r="IY16" s="115" t="s">
+        <v>11</v>
+      </c>
+      <c r="IZ16" s="115" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="17" spans="1:253" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="1:260" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="92">
         <v>14</v>
       </c>
@@ -28390,8 +29738,26 @@
       <c r="IS17" s="115" t="s">
         <v>3139</v>
       </c>
+      <c r="IT17" s="115" t="s">
+        <v>3866</v>
+      </c>
+      <c r="IU17" s="115" t="s">
+        <v>3878</v>
+      </c>
+      <c r="IV17" s="115" t="s">
+        <v>19</v>
+      </c>
+      <c r="IX17" s="115" t="s">
+        <v>819</v>
+      </c>
+      <c r="IY17" s="115" t="s">
+        <v>19</v>
+      </c>
+      <c r="IZ17" s="115" t="s">
+        <v>19</v>
+      </c>
     </row>
-    <row r="18" spans="1:253" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="1:260" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="92">
         <v>15</v>
       </c>
@@ -29147,8 +30513,26 @@
       <c r="IS18" s="115" t="s">
         <v>3851</v>
       </c>
+      <c r="IT18" s="115" t="s">
+        <v>3867</v>
+      </c>
+      <c r="IU18" s="115" t="s">
+        <v>3879</v>
+      </c>
+      <c r="IV18" s="115" t="s">
+        <v>3896</v>
+      </c>
+      <c r="IX18" s="115" t="s">
+        <v>3974</v>
+      </c>
+      <c r="IY18" s="115" t="s">
+        <v>3986</v>
+      </c>
+      <c r="IZ18" s="115" t="s">
+        <v>3986</v>
+      </c>
     </row>
-    <row r="19" spans="1:253" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" spans="1:260" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="92">
         <v>16</v>
       </c>
@@ -29904,8 +31288,26 @@
       <c r="IS19" s="115" t="s">
         <v>3852</v>
       </c>
+      <c r="IT19" s="115">
+        <v>2005</v>
+      </c>
+      <c r="IU19" s="115">
+        <v>2014</v>
+      </c>
+      <c r="IV19" s="115" t="s">
+        <v>3897</v>
+      </c>
+      <c r="IX19" s="115" t="s">
+        <v>3975</v>
+      </c>
+      <c r="IY19" s="115">
+        <v>2016</v>
+      </c>
+      <c r="IZ19" s="115">
+        <v>2015</v>
+      </c>
     </row>
-    <row r="20" spans="1:253" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="20" spans="1:260" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="92">
         <v>17</v>
       </c>
@@ -30661,8 +32063,26 @@
       <c r="IS20" s="115" t="s">
         <v>3853</v>
       </c>
+      <c r="IT20" s="115" t="s">
+        <v>1871</v>
+      </c>
+      <c r="IU20" s="115" t="s">
+        <v>1871</v>
+      </c>
+      <c r="IV20" s="115" t="s">
+        <v>1145</v>
+      </c>
+      <c r="IX20" s="115" t="s">
+        <v>3974</v>
+      </c>
+      <c r="IY20" s="115" t="s">
+        <v>2679</v>
+      </c>
+      <c r="IZ20" s="115" t="s">
+        <v>2679</v>
+      </c>
     </row>
-    <row r="21" spans="1:253" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="21" spans="1:260" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="92">
         <v>18</v>
       </c>
@@ -31414,8 +32834,26 @@
       <c r="IS21" s="115" t="s">
         <v>3854</v>
       </c>
+      <c r="IT21" s="115" t="s">
+        <v>3868</v>
+      </c>
+      <c r="IU21" s="115" t="s">
+        <v>3880</v>
+      </c>
+      <c r="IV21" s="115" t="s">
+        <v>3898</v>
+      </c>
+      <c r="IX21" s="159" t="s">
+        <v>3976</v>
+      </c>
+      <c r="IY21" s="115" t="s">
+        <v>3987</v>
+      </c>
+      <c r="IZ21" s="115" t="s">
+        <v>3999</v>
+      </c>
     </row>
-    <row r="22" spans="1:253" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="22" spans="1:260" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="92">
         <v>19</v>
       </c>
@@ -32173,8 +33611,26 @@
       <c r="IS22" s="115" t="s">
         <v>3855</v>
       </c>
+      <c r="IT22" s="115" t="s">
+        <v>3869</v>
+      </c>
+      <c r="IU22" s="115" t="s">
+        <v>3881</v>
+      </c>
+      <c r="IV22" s="115" t="s">
+        <v>3899</v>
+      </c>
+      <c r="IX22" s="115" t="s">
+        <v>3977</v>
+      </c>
+      <c r="IY22" s="115" t="s">
+        <v>3992</v>
+      </c>
+      <c r="IZ22" s="115" t="s">
+        <v>4000</v>
+      </c>
     </row>
-    <row r="23" spans="1:253" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="23" spans="1:260" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="92">
         <v>20</v>
       </c>
@@ -32932,8 +34388,26 @@
       <c r="IS23" s="115" t="s">
         <v>24</v>
       </c>
+      <c r="IT23" s="115" t="s">
+        <v>24</v>
+      </c>
+      <c r="IU23" s="115" t="s">
+        <v>24</v>
+      </c>
+      <c r="IV23" s="115" t="s">
+        <v>24</v>
+      </c>
+      <c r="IX23" s="115" t="s">
+        <v>24</v>
+      </c>
+      <c r="IY23" s="115" t="s">
+        <v>24</v>
+      </c>
+      <c r="IZ23" s="115" t="s">
+        <v>24</v>
+      </c>
     </row>
-    <row r="24" spans="1:253" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="1:260" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="92">
         <v>21</v>
       </c>
@@ -33691,8 +35165,26 @@
       <c r="IS24" s="115">
         <v>92</v>
       </c>
+      <c r="IT24" s="159">
+        <v>308</v>
+      </c>
+      <c r="IU24" s="115">
+        <v>192</v>
+      </c>
+      <c r="IV24" s="115">
+        <v>21345</v>
+      </c>
+      <c r="IX24" s="263">
+        <v>6</v>
+      </c>
+      <c r="IY24" s="115">
+        <v>63</v>
+      </c>
+      <c r="IZ24" s="115">
+        <v>63</v>
+      </c>
     </row>
-    <row r="25" spans="1:253" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" spans="1:260" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="92">
         <v>22</v>
       </c>
@@ -34443,8 +35935,26 @@
       <c r="IS25" s="159" t="s">
         <v>3856</v>
       </c>
+      <c r="IT25" s="217" t="s">
+        <v>3870</v>
+      </c>
+      <c r="IU25" s="217" t="s">
+        <v>3882</v>
+      </c>
+      <c r="IV25" s="159" t="s">
+        <v>3900</v>
+      </c>
+      <c r="IX25" s="159" t="s">
+        <v>3978</v>
+      </c>
+      <c r="IY25" s="159" t="s">
+        <v>3993</v>
+      </c>
+      <c r="IZ25" s="159" t="s">
+        <v>4001</v>
+      </c>
     </row>
-    <row r="26" spans="1:253" s="68" customFormat="1" ht="13.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="26" spans="1:260" s="68" customFormat="1" ht="13.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="92">
         <v>23</v>
       </c>
@@ -35204,8 +36714,26 @@
       <c r="IS26" s="159" t="s">
         <v>698</v>
       </c>
+      <c r="IT26" s="159" t="s">
+        <v>696</v>
+      </c>
+      <c r="IU26" s="159" t="s">
+        <v>696</v>
+      </c>
+      <c r="IV26" s="159" t="s">
+        <v>696</v>
+      </c>
+      <c r="IX26" s="159" t="s">
+        <v>1697</v>
+      </c>
+      <c r="IY26" s="159" t="s">
+        <v>696</v>
+      </c>
+      <c r="IZ26" s="159" t="s">
+        <v>696</v>
+      </c>
     </row>
-    <row r="27" spans="1:253" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="27" spans="1:260" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="92">
         <v>24</v>
       </c>
@@ -35963,8 +37491,26 @@
       <c r="IS27" s="159">
         <v>2</v>
       </c>
+      <c r="IT27" s="159">
+        <v>7</v>
+      </c>
+      <c r="IU27" s="159">
+        <v>7</v>
+      </c>
+      <c r="IV27" s="159">
+        <v>7</v>
+      </c>
+      <c r="IX27" s="159">
+        <v>28</v>
+      </c>
+      <c r="IY27" s="159">
+        <v>7</v>
+      </c>
+      <c r="IZ27" s="159">
+        <v>7</v>
+      </c>
     </row>
-    <row r="28" spans="1:253" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="28" spans="1:260" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="92">
         <v>25</v>
       </c>
@@ -36720,8 +38266,26 @@
       <c r="IS28" s="159" t="s">
         <v>696</v>
       </c>
+      <c r="IT28" s="159" t="s">
+        <v>1033</v>
+      </c>
+      <c r="IU28" s="159" t="s">
+        <v>1033</v>
+      </c>
+      <c r="IV28" s="159" t="s">
+        <v>1033</v>
+      </c>
+      <c r="IX28" s="159" t="s">
+        <v>1657</v>
+      </c>
+      <c r="IY28" s="184" t="s">
+        <v>698</v>
+      </c>
+      <c r="IZ28" s="184" t="s">
+        <v>698</v>
+      </c>
     </row>
-    <row r="29" spans="1:253" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="29" spans="1:260" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" s="92">
         <v>26</v>
       </c>
@@ -37477,8 +39041,26 @@
       <c r="IS29" s="182">
         <v>7</v>
       </c>
+      <c r="IT29" s="159">
+        <v>4</v>
+      </c>
+      <c r="IU29" s="159">
+        <v>4</v>
+      </c>
+      <c r="IV29" s="159">
+        <v>4</v>
+      </c>
+      <c r="IX29" s="184">
+        <v>28</v>
+      </c>
+      <c r="IY29" s="184">
+        <v>2</v>
+      </c>
+      <c r="IZ29" s="184">
+        <v>2</v>
+      </c>
     </row>
-    <row r="30" spans="1:253" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="30" spans="1:260" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="92">
         <v>27</v>
       </c>
@@ -38234,8 +39816,26 @@
       <c r="IS30" s="159" t="s">
         <v>704</v>
       </c>
+      <c r="IT30" s="159" t="s">
+        <v>1034</v>
+      </c>
+      <c r="IU30" s="159" t="s">
+        <v>1034</v>
+      </c>
+      <c r="IV30" s="159" t="s">
+        <v>1034</v>
+      </c>
+      <c r="IX30" s="159" t="s">
+        <v>696</v>
+      </c>
+      <c r="IY30" s="184" t="s">
+        <v>702</v>
+      </c>
+      <c r="IZ30" s="184" t="s">
+        <v>702</v>
+      </c>
     </row>
-    <row r="31" spans="1:253" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="31" spans="1:260" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="92">
         <v>28</v>
       </c>
@@ -38991,8 +40591,26 @@
       <c r="IS31" s="159">
         <v>9</v>
       </c>
+      <c r="IT31" s="184">
+        <v>20</v>
+      </c>
+      <c r="IU31" s="184">
+        <v>20</v>
+      </c>
+      <c r="IV31" s="184">
+        <v>20</v>
+      </c>
+      <c r="IX31" s="184">
+        <v>7</v>
+      </c>
+      <c r="IY31" s="184">
+        <v>3</v>
+      </c>
+      <c r="IZ31" s="184">
+        <v>3</v>
+      </c>
     </row>
-    <row r="32" spans="1:253" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="32" spans="1:260" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="92">
         <v>29</v>
       </c>
@@ -39748,8 +41366,26 @@
       <c r="IS32" s="184" t="s">
         <v>849</v>
       </c>
+      <c r="IT32" s="184" t="s">
+        <v>698</v>
+      </c>
+      <c r="IU32" s="184" t="s">
+        <v>698</v>
+      </c>
+      <c r="IV32" s="184" t="s">
+        <v>698</v>
+      </c>
+      <c r="IX32" s="159" t="s">
+        <v>697</v>
+      </c>
+      <c r="IY32" s="159" t="s">
+        <v>699</v>
+      </c>
+      <c r="IZ32" s="159" t="s">
+        <v>697</v>
+      </c>
     </row>
-    <row r="33" spans="1:253" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="33" spans="1:260" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="92">
         <v>30</v>
       </c>
@@ -40505,8 +42141,26 @@
       <c r="IS33" s="159">
         <v>4</v>
       </c>
+      <c r="IT33" s="184">
+        <v>2</v>
+      </c>
+      <c r="IU33" s="184">
+        <v>2</v>
+      </c>
+      <c r="IV33" s="184">
+        <v>2</v>
+      </c>
+      <c r="IX33" s="159">
+        <v>6</v>
+      </c>
+      <c r="IY33" s="159">
+        <v>6</v>
+      </c>
+      <c r="IZ33" s="159">
+        <v>6</v>
+      </c>
     </row>
-    <row r="34" spans="1:253" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="34" spans="1:260" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="92">
         <v>31</v>
       </c>
@@ -41262,8 +42916,26 @@
       <c r="IS34" s="184" t="s">
         <v>11</v>
       </c>
+      <c r="IT34" s="184" t="s">
+        <v>702</v>
+      </c>
+      <c r="IU34" s="184" t="s">
+        <v>702</v>
+      </c>
+      <c r="IV34" s="184" t="s">
+        <v>702</v>
+      </c>
+      <c r="IX34" s="159" t="s">
+        <v>698</v>
+      </c>
+      <c r="IY34" s="159" t="s">
+        <v>700</v>
+      </c>
+      <c r="IZ34" s="159" t="s">
+        <v>2179</v>
+      </c>
     </row>
-    <row r="35" spans="1:253" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="35" spans="1:260" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="92">
         <v>32</v>
       </c>
@@ -42019,8 +43691,26 @@
       <c r="IS35" s="184" t="s">
         <v>11</v>
       </c>
+      <c r="IT35" s="184">
+        <v>3</v>
+      </c>
+      <c r="IU35" s="184">
+        <v>3</v>
+      </c>
+      <c r="IV35" s="184">
+        <v>3</v>
+      </c>
+      <c r="IX35" s="184">
+        <v>2</v>
+      </c>
+      <c r="IY35" s="184">
+        <v>6</v>
+      </c>
+      <c r="IZ35" s="159">
+        <v>88</v>
+      </c>
     </row>
-    <row r="36" spans="1:253" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="36" spans="1:260" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="92">
         <v>33</v>
       </c>
@@ -42776,8 +44466,26 @@
       <c r="IS36" s="159" t="s">
         <v>11</v>
       </c>
+      <c r="IT36" s="159" t="s">
+        <v>699</v>
+      </c>
+      <c r="IU36" s="159" t="s">
+        <v>699</v>
+      </c>
+      <c r="IV36" s="159" t="s">
+        <v>699</v>
+      </c>
+      <c r="IX36" s="159" t="s">
+        <v>702</v>
+      </c>
+      <c r="IY36" s="159" t="s">
+        <v>2179</v>
+      </c>
+      <c r="IZ36" s="159" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="37" spans="1:253" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="37" spans="1:260" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="92">
         <v>34</v>
       </c>
@@ -43533,8 +45241,26 @@
       <c r="IS37" s="159" t="s">
         <v>11</v>
       </c>
+      <c r="IT37" s="159">
+        <v>6</v>
+      </c>
+      <c r="IU37" s="159">
+        <v>6</v>
+      </c>
+      <c r="IV37" s="159">
+        <v>6</v>
+      </c>
+      <c r="IX37" s="159">
+        <v>3</v>
+      </c>
+      <c r="IY37" s="159">
+        <v>88</v>
+      </c>
+      <c r="IZ37" s="159" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="38" spans="1:253" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="38" spans="1:260" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" s="92">
         <v>35</v>
       </c>
@@ -44290,8 +46016,26 @@
       <c r="IS38" s="159" t="s">
         <v>11</v>
       </c>
+      <c r="IT38" s="159" t="s">
+        <v>700</v>
+      </c>
+      <c r="IU38" s="159" t="s">
+        <v>700</v>
+      </c>
+      <c r="IV38" s="159" t="s">
+        <v>700</v>
+      </c>
+      <c r="IX38" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IY38" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IZ38" s="159" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="39" spans="1:253" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="39" spans="1:260" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="92">
         <v>36</v>
       </c>
@@ -45047,8 +46791,26 @@
       <c r="IS39" s="159" t="s">
         <v>11</v>
       </c>
+      <c r="IT39" s="184">
+        <v>6</v>
+      </c>
+      <c r="IU39" s="184">
+        <v>6</v>
+      </c>
+      <c r="IV39" s="184">
+        <v>6</v>
+      </c>
+      <c r="IX39" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IY39" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IZ39" s="159" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="40" spans="1:253" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="40" spans="1:260" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" s="92">
         <v>37</v>
       </c>
@@ -45804,8 +47566,26 @@
       <c r="IS40" s="159" t="s">
         <v>11</v>
       </c>
+      <c r="IT40" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IU40" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IV40" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IX40" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IY40" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IZ40" s="159" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="41" spans="1:253" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="41" spans="1:260" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A41" s="92">
         <v>38</v>
       </c>
@@ -46561,8 +48341,26 @@
       <c r="IS41" s="159" t="s">
         <v>11</v>
       </c>
+      <c r="IT41" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IU41" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IV41" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IX41" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IY41" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IZ41" s="159" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="42" spans="1:253" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="42" spans="1:260" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" s="92">
         <v>39</v>
       </c>
@@ -47318,8 +49116,26 @@
       <c r="IS42" s="159" t="s">
         <v>11</v>
       </c>
+      <c r="IT42" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IU42" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IV42" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IX42" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IY42" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IZ42" s="159" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="43" spans="1:253" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="43" spans="1:260" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" s="92">
         <v>40</v>
       </c>
@@ -48075,8 +49891,26 @@
       <c r="IS43" s="159" t="s">
         <v>11</v>
       </c>
+      <c r="IT43" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IU43" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IV43" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IX43" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IY43" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IZ43" s="159" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="44" spans="1:253" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="44" spans="1:260" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" s="92">
         <v>41</v>
       </c>
@@ -48832,8 +50666,26 @@
       <c r="IS44" s="159" t="s">
         <v>11</v>
       </c>
+      <c r="IT44" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IU44" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IV44" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IX44" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IY44" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IZ44" s="159" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="45" spans="1:253" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="45" spans="1:260" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" s="92">
         <v>42</v>
       </c>
@@ -49589,8 +51441,26 @@
       <c r="IS45" s="159" t="s">
         <v>11</v>
       </c>
+      <c r="IT45" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IU45" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IV45" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IX45" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IY45" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IZ45" s="159" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="46" spans="1:253" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="46" spans="1:260" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" s="92">
         <v>43</v>
       </c>
@@ -50346,8 +52216,26 @@
       <c r="IS46" s="159" t="s">
         <v>11</v>
       </c>
+      <c r="IT46" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IU46" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IV46" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IX46" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IY46" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IZ46" s="159" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="47" spans="1:253" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="47" spans="1:260" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" s="92">
         <v>44</v>
       </c>
@@ -51103,8 +52991,26 @@
       <c r="IS47" s="159" t="s">
         <v>11</v>
       </c>
+      <c r="IT47" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IU47" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IV47" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IX47" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IY47" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IZ47" s="159" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="48" spans="1:253" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="48" spans="1:260" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" s="92">
         <v>45</v>
       </c>
@@ -51860,8 +53766,26 @@
       <c r="IS48" s="159" t="s">
         <v>11</v>
       </c>
+      <c r="IT48" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IU48" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IV48" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IX48" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IY48" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IZ48" s="159" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="49" spans="1:253" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="49" spans="1:260" s="68" customFormat="1" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" s="92">
         <v>46</v>
       </c>
@@ -52617,8 +54541,26 @@
       <c r="IS49" s="159" t="s">
         <v>11</v>
       </c>
+      <c r="IT49" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IU49" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IV49" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IX49" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IY49" s="159" t="s">
+        <v>11</v>
+      </c>
+      <c r="IZ49" s="159" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="50" spans="1:253" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="50" spans="1:260" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" s="92">
         <v>47</v>
       </c>
@@ -53376,8 +55318,26 @@
       <c r="IS50" s="115" t="s">
         <v>2229</v>
       </c>
+      <c r="IT50" s="115" t="s">
+        <v>3776</v>
+      </c>
+      <c r="IU50" s="115" t="s">
+        <v>3776</v>
+      </c>
+      <c r="IV50" s="115" t="s">
+        <v>3776</v>
+      </c>
+      <c r="IX50" s="159" t="s">
+        <v>3979</v>
+      </c>
+      <c r="IY50" s="115" t="s">
+        <v>3988</v>
+      </c>
+      <c r="IZ50" s="115" t="s">
+        <v>4002</v>
+      </c>
     </row>
-    <row r="51" spans="1:253" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="51" spans="1:260" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" s="92">
         <v>48</v>
       </c>
@@ -54135,8 +56095,26 @@
       <c r="IS51" s="115" t="s">
         <v>3857</v>
       </c>
+      <c r="IT51" s="115" t="s">
+        <v>3871</v>
+      </c>
+      <c r="IU51" s="115" t="s">
+        <v>3883</v>
+      </c>
+      <c r="IV51" s="159" t="s">
+        <v>3901</v>
+      </c>
+      <c r="IX51" s="159" t="s">
+        <v>3980</v>
+      </c>
+      <c r="IY51" s="115" t="s">
+        <v>3989</v>
+      </c>
+      <c r="IZ51" s="115" t="s">
+        <v>4003</v>
+      </c>
     </row>
-    <row r="52" spans="1:253" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="52" spans="1:260" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A52" s="92">
         <v>49</v>
       </c>
@@ -54894,8 +56872,26 @@
       <c r="IS52" s="115" t="s">
         <v>3858</v>
       </c>
+      <c r="IT52" s="159" t="s">
+        <v>3778</v>
+      </c>
+      <c r="IU52" s="115" t="s">
+        <v>3778</v>
+      </c>
+      <c r="IV52" s="115" t="s">
+        <v>3778</v>
+      </c>
+      <c r="IX52" s="159" t="s">
+        <v>3619</v>
+      </c>
+      <c r="IY52" s="115" t="s">
+        <v>3990</v>
+      </c>
+      <c r="IZ52" s="115" t="s">
+        <v>4004</v>
+      </c>
     </row>
-    <row r="53" spans="1:253" ht="14.05" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:260" ht="14.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A53" s="92">
         <v>50</v>
       </c>
@@ -55655,8 +57651,26 @@
       <c r="IS53" s="183" t="s">
         <v>206</v>
       </c>
+      <c r="IT53" s="183" t="s">
+        <v>206</v>
+      </c>
+      <c r="IU53" s="185" t="s">
+        <v>206</v>
+      </c>
+      <c r="IV53" s="185" t="s">
+        <v>206</v>
+      </c>
+      <c r="IX53" s="183" t="s">
+        <v>206</v>
+      </c>
+      <c r="IY53" s="185" t="s">
+        <v>206</v>
+      </c>
+      <c r="IZ53" s="185" t="s">
+        <v>206</v>
+      </c>
     </row>
-    <row r="54" spans="1:253" ht="13.8" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:260" ht="13.8" x14ac:dyDescent="0.45">
       <c r="A54" s="92">
         <v>51</v>
       </c>
@@ -56414,8 +58428,26 @@
       <c r="IS54" s="115" t="s">
         <v>61</v>
       </c>
+      <c r="IT54" s="183" t="s">
+        <v>61</v>
+      </c>
+      <c r="IU54" s="185" t="s">
+        <v>61</v>
+      </c>
+      <c r="IV54" s="185" t="s">
+        <v>61</v>
+      </c>
+      <c r="IX54" s="159" t="s">
+        <v>2651</v>
+      </c>
+      <c r="IY54" s="185" t="s">
+        <v>3109</v>
+      </c>
+      <c r="IZ54" s="185" t="s">
+        <v>3109</v>
+      </c>
     </row>
-    <row r="55" spans="1:253" ht="13.8" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:260" ht="13.8" x14ac:dyDescent="0.45">
       <c r="A55" s="92">
         <v>52</v>
       </c>
@@ -57173,8 +59205,26 @@
       <c r="IS55" s="159" t="s">
         <v>3859</v>
       </c>
+      <c r="IT55" s="183" t="s">
+        <v>3872</v>
+      </c>
+      <c r="IU55" s="185" t="s">
+        <v>3884</v>
+      </c>
+      <c r="IV55" s="185" t="s">
+        <v>3243</v>
+      </c>
+      <c r="IX55" s="159" t="s">
+        <v>3981</v>
+      </c>
+      <c r="IY55" s="185" t="s">
+        <v>40</v>
+      </c>
+      <c r="IZ55" s="185" t="s">
+        <v>40</v>
+      </c>
     </row>
-    <row r="56" spans="1:253" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="56" spans="1:260" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A56" s="92">
         <v>53</v>
       </c>
@@ -57930,8 +59980,26 @@
       <c r="IS56" s="159" t="s">
         <v>3860</v>
       </c>
+      <c r="IT56" s="183" t="s">
+        <v>3873</v>
+      </c>
+      <c r="IU56" s="185" t="s">
+        <v>3885</v>
+      </c>
+      <c r="IV56" s="185" t="s">
+        <v>3902</v>
+      </c>
+      <c r="IX56" s="215" t="s">
+        <v>3981</v>
+      </c>
+      <c r="IY56" s="185" t="s">
+        <v>3991</v>
+      </c>
+      <c r="IZ56" s="185" t="s">
+        <v>3991</v>
+      </c>
     </row>
-    <row r="57" spans="1:253" ht="13.8" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:260" ht="13.8" x14ac:dyDescent="0.45">
       <c r="A57" s="92">
         <v>54</v>
       </c>
@@ -58689,8 +60757,26 @@
       <c r="IS57" s="159" t="s">
         <v>3861</v>
       </c>
+      <c r="IT57" s="159" t="s">
+        <v>3874</v>
+      </c>
+      <c r="IU57" s="115" t="s">
+        <v>3886</v>
+      </c>
+      <c r="IV57" s="115" t="s">
+        <v>3903</v>
+      </c>
+      <c r="IX57" s="159" t="s">
+        <v>3981</v>
+      </c>
+      <c r="IY57" s="115" t="s">
+        <v>3671</v>
+      </c>
+      <c r="IZ57" s="115" t="s">
+        <v>3671</v>
+      </c>
     </row>
-    <row r="58" spans="1:253" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="58" spans="1:260" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" s="92">
         <v>55</v>
       </c>
@@ -59419,8 +61505,26 @@
       <c r="IS58" s="159" t="s">
         <v>3860</v>
       </c>
+      <c r="IT58" s="183" t="s">
+        <v>3873</v>
+      </c>
+      <c r="IU58" s="185" t="s">
+        <v>3887</v>
+      </c>
+      <c r="IV58" s="185" t="s">
+        <v>3904</v>
+      </c>
+      <c r="IX58" s="215" t="s">
+        <v>3981</v>
+      </c>
+      <c r="IY58" s="185" t="s">
+        <v>3991</v>
+      </c>
+      <c r="IZ58" s="185" t="s">
+        <v>3991</v>
+      </c>
     </row>
-    <row r="59" spans="1:253" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="59" spans="1:260" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" s="92">
         <v>56</v>
       </c>
@@ -60178,8 +62282,26 @@
       <c r="IS59" s="159" t="s">
         <v>3860</v>
       </c>
+      <c r="IT59" s="183" t="s">
+        <v>3873</v>
+      </c>
+      <c r="IU59" s="185" t="s">
+        <v>3887</v>
+      </c>
+      <c r="IV59" s="185" t="s">
+        <v>3904</v>
+      </c>
+      <c r="IX59" s="215" t="s">
+        <v>3981</v>
+      </c>
+      <c r="IY59" s="185" t="s">
+        <v>3991</v>
+      </c>
+      <c r="IZ59" s="185" t="s">
+        <v>3991</v>
+      </c>
     </row>
-    <row r="60" spans="1:253" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="60" spans="1:260" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A60" s="92">
         <v>57</v>
       </c>
@@ -60937,8 +63059,26 @@
       <c r="IS60" s="182">
         <v>1</v>
       </c>
+      <c r="IT60" s="182">
+        <v>1</v>
+      </c>
+      <c r="IU60" s="184">
+        <v>1</v>
+      </c>
+      <c r="IV60" s="184">
+        <v>1</v>
+      </c>
+      <c r="IX60" s="65">
+        <v>1</v>
+      </c>
+      <c r="IY60" s="184">
+        <v>1</v>
+      </c>
+      <c r="IZ60" s="184">
+        <v>1</v>
+      </c>
     </row>
-    <row r="61" spans="1:253" ht="14.05" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:260" ht="14.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A61" s="92">
         <v>58</v>
       </c>
@@ -61696,8 +63836,26 @@
       <c r="IS61" s="157">
         <v>46028</v>
       </c>
+      <c r="IT61" s="221">
+        <v>46029</v>
+      </c>
+      <c r="IU61" s="157">
+        <v>46028</v>
+      </c>
+      <c r="IV61" s="157">
+        <v>45823</v>
+      </c>
+      <c r="IX61" s="157">
+        <v>46031</v>
+      </c>
+      <c r="IY61" s="157">
+        <v>46031</v>
+      </c>
+      <c r="IZ61" s="157">
+        <v>46031</v>
+      </c>
     </row>
-    <row r="62" spans="1:253" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="62" spans="1:260" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A62" s="92">
         <v>59</v>
       </c>
@@ -62455,8 +64613,26 @@
       <c r="IS62" s="157">
         <v>46028</v>
       </c>
+      <c r="IT62" s="221">
+        <v>46029</v>
+      </c>
+      <c r="IU62" s="157">
+        <v>46028</v>
+      </c>
+      <c r="IV62" s="157">
+        <v>45825</v>
+      </c>
+      <c r="IX62" s="157">
+        <v>46031</v>
+      </c>
+      <c r="IY62" s="157">
+        <v>46031</v>
+      </c>
+      <c r="IZ62" s="157">
+        <v>46031</v>
+      </c>
     </row>
-    <row r="63" spans="1:253" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="63" spans="1:260" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A63" s="92">
         <v>60</v>
       </c>
@@ -63214,8 +65390,26 @@
       <c r="IS63" s="115" t="s">
         <v>30</v>
       </c>
+      <c r="IT63" s="159" t="s">
+        <v>30</v>
+      </c>
+      <c r="IU63" s="115" t="s">
+        <v>30</v>
+      </c>
+      <c r="IV63" s="115" t="s">
+        <v>30</v>
+      </c>
+      <c r="IX63" s="169" t="s">
+        <v>30</v>
+      </c>
+      <c r="IY63" s="115" t="s">
+        <v>30</v>
+      </c>
+      <c r="IZ63" s="115" t="s">
+        <v>30</v>
+      </c>
     </row>
-    <row r="64" spans="1:253" ht="14.4" x14ac:dyDescent="0.55000000000000004">
+    <row r="64" spans="1:260" ht="14.4" x14ac:dyDescent="0.55000000000000004">
       <c r="A64" s="92">
         <v>61</v>
       </c>
@@ -63972,6 +66166,24 @@
       </c>
       <c r="IS64" s="115" t="s">
         <v>3165</v>
+      </c>
+      <c r="IT64" s="159" t="s">
+        <v>3875</v>
+      </c>
+      <c r="IU64" s="217" t="s">
+        <v>3888</v>
+      </c>
+      <c r="IV64" s="159" t="s">
+        <v>3900</v>
+      </c>
+      <c r="IX64" s="185" t="s">
+        <v>3580</v>
+      </c>
+      <c r="IY64" s="159" t="s">
+        <v>3994</v>
+      </c>
+      <c r="IZ64" s="159" t="s">
+        <v>4005</v>
       </c>
     </row>
     <row r="65" spans="1:263" ht="14.4" x14ac:dyDescent="0.55000000000000004">
@@ -64435,6 +66647,24 @@
       <c r="IS65" s="157">
         <v>46028</v>
       </c>
+      <c r="IT65" s="221">
+        <v>46029</v>
+      </c>
+      <c r="IU65" s="157">
+        <v>46028</v>
+      </c>
+      <c r="IV65" s="221">
+        <v>46029</v>
+      </c>
+      <c r="IX65" s="157">
+        <v>46031</v>
+      </c>
+      <c r="IY65" s="157">
+        <v>46031</v>
+      </c>
+      <c r="IZ65" s="157">
+        <v>46031</v>
+      </c>
     </row>
     <row r="66" spans="1:263" ht="13.8" x14ac:dyDescent="0.45">
       <c r="A66" s="92">
@@ -64893,6 +67123,24 @@
         <v>30</v>
       </c>
       <c r="IS66" s="169" t="s">
+        <v>30</v>
+      </c>
+      <c r="IT66" s="159" t="s">
+        <v>30</v>
+      </c>
+      <c r="IU66" s="115" t="s">
+        <v>30</v>
+      </c>
+      <c r="IV66" s="115" t="s">
+        <v>30</v>
+      </c>
+      <c r="IX66" s="169" t="s">
+        <v>30</v>
+      </c>
+      <c r="IY66" s="115" t="s">
+        <v>30</v>
+      </c>
+      <c r="IZ66" s="115" t="s">
         <v>30</v>
       </c>
     </row>
@@ -65055,6 +67303,12 @@
       <c r="IM67" s="156"/>
       <c r="IQ67" s="206"/>
       <c r="IR67" s="156"/>
+      <c r="IT67" s="237"/>
+      <c r="IU67" s="206"/>
+      <c r="IV67" s="206"/>
+      <c r="IX67" s="156"/>
+      <c r="IY67" s="206"/>
+      <c r="IZ67" s="206"/>
     </row>
     <row r="68" spans="1:263" ht="13.8" x14ac:dyDescent="0.45">
       <c r="A68" s="92">
@@ -65142,7 +67396,21 @@
       <c r="HK68" s="185"/>
       <c r="HL68" s="156"/>
       <c r="HM68" s="169"/>
+      <c r="IK68" s="237" t="s">
+        <v>3876</v>
+      </c>
       <c r="IR68" s="156"/>
+      <c r="IT68" s="237" t="s">
+        <v>3876</v>
+      </c>
+      <c r="IU68" s="237" t="s">
+        <v>3876</v>
+      </c>
+      <c r="IV68" s="237" t="s">
+        <v>3876</v>
+      </c>
+      <c r="IX68" s="156"/>
+      <c r="IY68" s="206"/>
     </row>
     <row r="69" spans="1:263" ht="13.8" x14ac:dyDescent="0.45">
       <c r="A69" s="92">
@@ -65198,6 +67466,9 @@
       <c r="HK69" s="185"/>
       <c r="HM69" s="156"/>
       <c r="IR69" s="156"/>
+      <c r="IU69" s="206"/>
+      <c r="IV69" s="206"/>
+      <c r="IY69" s="206"/>
     </row>
     <row r="70" spans="1:263" ht="13.8" x14ac:dyDescent="0.45">
       <c r="A70" s="92">
@@ -65240,6 +67511,7 @@
       <c r="GW70" s="206"/>
       <c r="HK70" s="156"/>
       <c r="IR70" s="156"/>
+      <c r="IV70" s="206"/>
     </row>
     <row r="71" spans="1:263" ht="13.8" x14ac:dyDescent="0.45">
       <c r="A71" s="92">

</xml_diff>